<commit_message>
Blueprint + proforma: Crew 1 equipment owned; Crew 2 rent-then-own path per item (Equipment plan tab, page 8)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LoK8Mi2K1W9PhhoHM3MdEb
</commit_message>
<xml_diff>
--- a/docs/Scag-Scapes-Proforma.xlsx
+++ b/docs/Scag-Scapes-Proforma.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Proforma 24 mo" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Unit economics" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Scenarios" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Sources &amp; notes" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Equipment plan" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Sources &amp; notes" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="285">
   <si>
     <t xml:space="preserve">Scag Scapes LLC - Growth Proforma - Assumptions</t>
   </si>
@@ -302,25 +303,85 @@
     <t xml:space="preserve">Left at $0 on purpose - terms to be agreed. Enter a number to see the effect.</t>
   </si>
   <si>
-    <t xml:space="preserve">CREW 2 STARTUP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipment purchase - mini excavator, trailer, tools ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Used 3.5-4 ton mini-ex ~$45-55K + dump trailer + hand tools. Alternative: rent at ~$2,000/mo (Home Depot live rate in the app) for the first 90 days.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Truck for Crew 2 ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Used 3/4-ton.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% financed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20% down.</t>
+    <t xml:space="preserve">CREW 2 EQUIPMENT - rent first, then own (Crew 1 already owns its trailer, skid steer and mini excavator)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mini excavator (3.5-4 ton, used) - purchase price ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used KX040 / 26G class. Crew 1's is owned; Crew 2 needs its own.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mini excavator - rental per month ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home Depot 4-week rate ~$1,700-2,000 (live in the app); Sunbelt/United quote-only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mini excavator - months rented before buying</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rent while Crew 2 proves itself; buy after it hits target twice. 0 = buy at start.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skid steer / CTL (used) - purchase price ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used T66 / 259D class.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skid steer - rental per month ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chain 4-week rate (rate card, CALL_TO_CONFIRM).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skid steer - months rented before buying</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dump trailer 7x14 (new) - purchase price ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trailers rent badly and hold value - buy at start.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dump trailer - rental per month ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dump trailer - months rented before buying</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 = buy at Crew 2 start.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Truck 3/4-ton (used) - purchase price ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Truck - rental per month ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not rented.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Truck - months rented before buying</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hand tools, laser, compactor, PPE, phones ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bought at start.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tools - rental per month ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tools - months rented before buying</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% financed on purchases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20% down on each purchase.</t>
   </si>
   <si>
     <t xml:space="preserve">Loan rate (APR)</t>
@@ -332,18 +393,6 @@
     <t xml:space="preserve">Loan term (months)</t>
   </si>
   <si>
-    <t xml:space="preserve">Rent instead of buy for first 3 months? (1 = yes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Safer: rent the mini-ex for months 7-9, buy when Crew 2 has hit target twice.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rental cost per month while renting ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Home Depot 3.5-4 ton ~$439/day, ~$1,700-2,000 4-week; app shows live.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hiring + training cost for Crew 2 (one-time $)</t>
   </si>
   <si>
@@ -482,10 +531,10 @@
     <t xml:space="preserve">Marketing - content, reviews, GBP, site</t>
   </si>
   <si>
-    <t xml:space="preserve">Crew 2 - rental (months before purchase) + hiring</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crew 2 - equipment + truck loan payment</t>
+    <t xml:space="preserve">Crew 2 - equipment rental (before purchase) + hiring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew 2 - equipment + truck loan payments</t>
   </si>
   <si>
     <t xml:space="preserve">Total overhead</t>
@@ -506,7 +555,7 @@
     <t xml:space="preserve">Cash out - direct costs + overhead</t>
   </si>
   <si>
-    <t xml:space="preserve">Cash out - Crew 2 down payment (equipment + truck)</t>
+    <t xml:space="preserve">Cash out - Crew 2 down payments (20% of each purchase)</t>
   </si>
   <si>
     <t xml:space="preserve">NET CASH FLOW</t>
@@ -686,6 +735,78 @@
     <t xml:space="preserve">Stretch: pricing power from reviews + Moasure proposals lifts $/LF to $46; 140 plan customers = the sellable recurring book.</t>
   </si>
   <si>
+    <t xml:space="preserve">Path to owning Crew 2's equipment - rent first, buy on proof</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew 1 already owns a big trailer, a skid steer and a mini excavator (no capex in this plan). Crew 2 needs its own set. Rent-to-prove, then buy; every date is driven by the Crew 2 start month on Assumptions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purchase price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rent / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Months rented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rent paid before buying</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purchase month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Down payment (20%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan payment / mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan paid off (month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Own-vs-rent break-even (months)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mini excavator (used)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skid steer / CTL (used)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dump trailer 7x14 (new)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Truck 3/4-ton (used)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tools, laser, compactor, PPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How to read it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Own-vs-rent break-even: purchase price / monthly rent. A mini-ex at $50,000 vs $2,000/month breaks even at 25 months of use - so anything Crew 2 will run for more than two years should be owned; the 3-month rental is insurance against Crew 2 not working out, not a long-term plan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The purchase month is the Crew 2 start month plus the months rented. Decision rule for pulling the trigger early or late: buy when Crew 2 has installed its target LF in two consecutive months; keep renting if it has not.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Down payments hit cash in the purchase month (Proforma: 'Cash out - Crew 2 down payments'); loan payments run 60 months from there. Rent paid before buying is money spent to de-risk the purchase - budgeted, not wasted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew 1's set is already owned: no purchases are modeled for it. Its existing payments, if any, sit in 'Existing truck / equipment payments' on Assumptions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time to full ownership of Crew 2's set: trailer, truck and tools on day one; mini-ex and skid steer bought in month start+3; all loans paid off 60 months after that (month 70 in the base case). Equity builds from the first payment; the machines outlast the loans.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sources and notes</t>
   </si>
   <si>
@@ -758,7 +879,7 @@
     <t xml:space="preserve">Model conventions</t>
   </si>
   <si>
-    <t xml:space="preserve">Revenue recognized in month of install; 30% deposit at signing, 90% of balance in month of completion, 10% the following month. Payroll burden 18% is an estimate - replace with actual workers' comp rate. No income tax modeled (pass-through LLC). Crew 2 equipment: rent 3 months then buy, 80% financed at 9% over 60 months.</t>
+    <t xml:space="preserve">Revenue recognized in month of install; 30% deposit at signing, 90% of balance in month of completion, 10% the following month. Payroll burden 18% is an estimate - replace with actual workers' comp rate. No income tax modeled (pass-through LLC). Crew 2 equipment: Crew 1 already owns its trailer, skid steer and mini excavator; Crew 2's mini-ex and skid steer are rented for 3 months then bought (80% financed, 9%, 60 months); trailer, truck and tools bought at start.</t>
   </si>
 </sst>
 </file>
@@ -928,7 +1049,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1047,6 +1168,14 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -1309,7 +1438,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -1863,7 +1992,7 @@
         <v>93</v>
       </c>
       <c r="B54" s="13" t="n">
-        <v>65000</v>
+        <v>50000</v>
       </c>
       <c r="C54" s="7" t="s">
         <v>94</v>
@@ -1874,7 +2003,7 @@
         <v>95</v>
       </c>
       <c r="B55" s="14" t="n">
-        <v>35000</v>
+        <v>2000</v>
       </c>
       <c r="C55" s="7" t="s">
         <v>96</v>
@@ -1884,8 +2013,8 @@
       <c r="A56" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B56" s="12" t="n">
-        <v>0.8</v>
+      <c r="B56" s="6" t="n">
+        <v>3</v>
       </c>
       <c r="C56" s="7" t="s">
         <v>98</v>
@@ -1895,8 +2024,8 @@
       <c r="A57" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B57" s="12" t="n">
-        <v>0.09</v>
+      <c r="B57" s="13" t="n">
+        <v>38000</v>
       </c>
       <c r="C57" s="7" t="s">
         <v>100</v>
@@ -1906,28 +2035,28 @@
       <c r="A58" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B58" s="10" t="n">
-        <v>60</v>
-      </c>
-      <c r="C58" s="7"/>
+      <c r="B58" s="14" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B59" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C59" s="7" t="s">
-        <v>103</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="C59" s="7"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
         <v>104</v>
       </c>
       <c r="B60" s="14" t="n">
-        <v>2000</v>
+        <v>9500</v>
       </c>
       <c r="C60" s="7" t="s">
         <v>105</v>
@@ -1938,10 +2067,119 @@
         <v>106</v>
       </c>
       <c r="B61" s="14" t="n">
+        <v>600</v>
+      </c>
+      <c r="C61" s="7"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B62" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B63" s="14" t="n">
+        <v>35000</v>
+      </c>
+      <c r="C63" s="7"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B64" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B65" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C65" s="7"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B66" s="14" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B67" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C67" s="7"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B68" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C68" s="7"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B69" s="12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C69" s="7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B70" s="12" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B71" s="10" t="n">
+        <v>60</v>
+      </c>
+      <c r="C71" s="7"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B72" s="14" t="n">
         <v>4500</v>
       </c>
-      <c r="C61" s="7" t="s">
-        <v>107</v>
+      <c r="C72" s="7" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1970,7 +2208,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2002,7 +2240,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2064,7 +2302,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="B4" s="16" t="n">
         <v>1</v>
@@ -2139,18 +2377,18 @@
         <v>24</v>
       </c>
       <c r="Z4" s="15" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="AA4" s="15" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="AB4" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>114</v>
+        <v>130</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -2182,7 +2420,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="B6" s="18" t="n">
         <f aca="false">MIN(Assumptions!$B$7,Assumptions!$B$6+(Assumptions!$B$7-Assumptions!$B$6)*(1-1)/5)</f>
@@ -2295,7 +2533,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="B7" s="18" t="n">
         <f aca="false">IF(1&lt;Assumptions!$B$8,0,MIN(Assumptions!$B$10,Assumptions!$B$9+(Assumptions!$B$10-Assumptions!$B$9)*(1-Assumptions!$B$8)/3))</f>
@@ -2408,7 +2646,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="B8" s="19" t="n">
         <f aca="false">B6+B7</f>
@@ -2521,7 +2759,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -2553,7 +2791,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="B10" s="18" t="n">
         <f aca="false">Assumptions!$B$34*IF(1&gt;=Assumptions!$B$8,Assumptions!$B$43,1)/Assumptions!$B$35</f>
@@ -2666,7 +2904,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="B11" s="18" t="n">
         <f aca="false">IF(1&gt;=2,Assumptions!$B$37*IF(1&gt;=Assumptions!$B$8,Assumptions!$B$43,1)/Assumptions!$B$38,0)</f>
@@ -2779,7 +3017,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="B12" s="18" t="n">
         <f aca="false">Assumptions!$B$40*(1+Assumptions!$B$41)^(1-1)</f>
@@ -2892,7 +3130,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="B13" s="19" t="n">
         <f aca="false">B10+B11+B12</f>
@@ -3005,7 +3243,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="B14" s="18" t="n">
         <f aca="false">B10*Assumptions!$B$36+B11*Assumptions!$B$39+B12*Assumptions!$B$42</f>
@@ -3118,7 +3356,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="B15" s="18" t="n">
         <f aca="false">B14*Assumptions!$B$11</f>
@@ -3231,7 +3469,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="B16" s="19" t="n">
         <f aca="false">MIN(B15+0,B8)</f>
@@ -3344,7 +3582,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
       <c r="B17" s="18" t="n">
         <f aca="false">MIN(B8*Assumptions!$B$12,MAX(0,B15+0-B16))</f>
@@ -3448,7 +3686,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="B18" s="20" t="n">
         <f aca="false">IF(B8=0,0,B16/B8)</f>
@@ -3552,7 +3790,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -3584,7 +3822,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="B20" s="21" t="n">
         <f aca="false">B16*Assumptions!$B$5</f>
@@ -3697,7 +3935,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
       <c r="B21" s="18" t="n">
         <f aca="false">IF(1&lt;Assumptions!$B$26,0,B16/Assumptions!$B$11*Assumptions!$B$23+IF(1&lt;=Assumptions!$B$26+11,Assumptions!$B$24*Assumptions!$B$25/12,0))</f>
@@ -3810,7 +4048,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="B22" s="18" t="n">
         <f aca="false">0+B21</f>
@@ -3914,7 +4152,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="B23" s="21" t="n">
         <f aca="false">B22/12/Assumptions!$B$22*Assumptions!$B$21</f>
@@ -4027,7 +4265,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="B24" s="22" t="n">
         <f aca="false">B20+B23</f>
@@ -4140,7 +4378,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -4172,7 +4410,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
       <c r="B26" s="21" t="n">
         <f aca="false">B20*Assumptions!$B$14</f>
@@ -4285,7 +4523,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="B27" s="21" t="n">
         <f aca="false">B20*Assumptions!$B$15</f>
@@ -4398,7 +4636,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="B28" s="21" t="n">
         <f aca="false">B22/12/Assumptions!$B$22*Assumptions!$B$27</f>
@@ -4511,7 +4749,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>138</v>
+        <v>154</v>
       </c>
       <c r="B29" s="22" t="n">
         <f aca="false">B26+B27+B28</f>
@@ -4624,7 +4862,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="B30" s="23" t="n">
         <f aca="false">B24-B29</f>
@@ -4737,7 +4975,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="s">
-        <v>140</v>
+        <v>156</v>
       </c>
       <c r="B31" s="20" t="n">
         <f aca="false">IF(B24=0,0,B30/B24)</f>
@@ -4841,7 +5079,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -4873,7 +5111,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="B33" s="21" t="n">
         <f aca="false">Assumptions!$B$46</f>
@@ -4986,7 +5224,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="B34" s="21" t="n">
         <f aca="false">Assumptions!$B$47</f>
@@ -5099,7 +5337,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="17" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
       <c r="B35" s="21" t="n">
         <f aca="false">Assumptions!$B$48</f>
@@ -5212,7 +5450,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="17" t="s">
-        <v>145</v>
+        <v>161</v>
       </c>
       <c r="B36" s="21" t="n">
         <f aca="false">Assumptions!$B$49</f>
@@ -5325,7 +5563,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="17" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
       <c r="B37" s="21" t="n">
         <f aca="false">Assumptions!$B$50</f>
@@ -5438,7 +5676,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="17" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="B38" s="21" t="n">
         <f aca="false">Assumptions!$B$51</f>
@@ -5551,7 +5789,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="17" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="B39" s="21" t="n">
         <f aca="false">Assumptions!$B$52</f>
@@ -5664,7 +5902,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="17" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="B40" s="21" t="n">
         <f aca="false">Assumptions!$B$34*IF(1&gt;=Assumptions!$B$8,Assumptions!$B$43,1)</f>
@@ -5777,7 +6015,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="17" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="B41" s="21" t="n">
         <f aca="false">IF(1&gt;=2,Assumptions!$B$37*IF(1&gt;=Assumptions!$B$8,Assumptions!$B$43,1),0)</f>
@@ -5890,7 +6128,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="17" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="B42" s="21" t="n">
         <f aca="false">Assumptions!$B$44</f>
@@ -6003,107 +6241,107 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="17" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="B43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,1&gt;=Assumptions!$B$8,1&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(1=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(1&gt;=Assumptions!$B$8,1&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(1&gt;=Assumptions!$B$8,1&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(1&gt;=Assumptions!$B$8,1&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(1&gt;=Assumptions!$B$8,1&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(1&gt;=Assumptions!$B$8,1&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(1=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="C43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,2&gt;=Assumptions!$B$8,2&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(2=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(2&gt;=Assumptions!$B$8,2&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(2&gt;=Assumptions!$B$8,2&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(2&gt;=Assumptions!$B$8,2&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(2&gt;=Assumptions!$B$8,2&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(2&gt;=Assumptions!$B$8,2&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(2=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="D43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,3&gt;=Assumptions!$B$8,3&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(3=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(3&gt;=Assumptions!$B$8,3&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(3&gt;=Assumptions!$B$8,3&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(3&gt;=Assumptions!$B$8,3&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(3&gt;=Assumptions!$B$8,3&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(3&gt;=Assumptions!$B$8,3&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(3=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="E43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,4&gt;=Assumptions!$B$8,4&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(4=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(4&gt;=Assumptions!$B$8,4&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(4&gt;=Assumptions!$B$8,4&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(4&gt;=Assumptions!$B$8,4&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(4&gt;=Assumptions!$B$8,4&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(4&gt;=Assumptions!$B$8,4&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(4=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="F43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,5&gt;=Assumptions!$B$8,5&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(5=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(5&gt;=Assumptions!$B$8,5&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(5&gt;=Assumptions!$B$8,5&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(5&gt;=Assumptions!$B$8,5&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(5&gt;=Assumptions!$B$8,5&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(5&gt;=Assumptions!$B$8,5&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(5=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="G43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,6&gt;=Assumptions!$B$8,6&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(6=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(6&gt;=Assumptions!$B$8,6&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(6&gt;=Assumptions!$B$8,6&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(6&gt;=Assumptions!$B$8,6&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(6&gt;=Assumptions!$B$8,6&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(6&gt;=Assumptions!$B$8,6&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(6=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="H43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,7&gt;=Assumptions!$B$8,7&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(7=Assumptions!$B$8,Assumptions!$B$61,0)</f>
-        <v>6500</v>
+        <f aca="false">IF(AND(7&gt;=Assumptions!$B$8,7&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(7&gt;=Assumptions!$B$8,7&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(7&gt;=Assumptions!$B$8,7&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(7&gt;=Assumptions!$B$8,7&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(7&gt;=Assumptions!$B$8,7&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(7=Assumptions!$B$8,Assumptions!$B$72,0)</f>
+        <v>8200</v>
       </c>
       <c r="I43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,8&gt;=Assumptions!$B$8,8&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(8=Assumptions!$B$8,Assumptions!$B$61,0)</f>
-        <v>2000</v>
+        <f aca="false">IF(AND(8&gt;=Assumptions!$B$8,8&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(8&gt;=Assumptions!$B$8,8&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(8&gt;=Assumptions!$B$8,8&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(8&gt;=Assumptions!$B$8,8&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(8&gt;=Assumptions!$B$8,8&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(8=Assumptions!$B$8,Assumptions!$B$72,0)</f>
+        <v>3700</v>
       </c>
       <c r="J43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,9&gt;=Assumptions!$B$8,9&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(9=Assumptions!$B$8,Assumptions!$B$61,0)</f>
-        <v>2000</v>
+        <f aca="false">IF(AND(9&gt;=Assumptions!$B$8,9&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(9&gt;=Assumptions!$B$8,9&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(9&gt;=Assumptions!$B$8,9&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(9&gt;=Assumptions!$B$8,9&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(9&gt;=Assumptions!$B$8,9&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(9=Assumptions!$B$8,Assumptions!$B$72,0)</f>
+        <v>3700</v>
       </c>
       <c r="K43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,10&gt;=Assumptions!$B$8,10&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(10=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(10&gt;=Assumptions!$B$8,10&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(10&gt;=Assumptions!$B$8,10&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(10&gt;=Assumptions!$B$8,10&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(10&gt;=Assumptions!$B$8,10&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(10&gt;=Assumptions!$B$8,10&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(10=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="L43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,11&gt;=Assumptions!$B$8,11&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(11=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(11&gt;=Assumptions!$B$8,11&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(11&gt;=Assumptions!$B$8,11&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(11&gt;=Assumptions!$B$8,11&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(11&gt;=Assumptions!$B$8,11&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(11&gt;=Assumptions!$B$8,11&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(11=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="M43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,12&gt;=Assumptions!$B$8,12&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(12=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(12&gt;=Assumptions!$B$8,12&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(12&gt;=Assumptions!$B$8,12&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(12&gt;=Assumptions!$B$8,12&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(12&gt;=Assumptions!$B$8,12&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(12&gt;=Assumptions!$B$8,12&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(12=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="N43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,13&gt;=Assumptions!$B$8,13&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(13=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(13&gt;=Assumptions!$B$8,13&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(13&gt;=Assumptions!$B$8,13&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(13&gt;=Assumptions!$B$8,13&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(13&gt;=Assumptions!$B$8,13&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(13&gt;=Assumptions!$B$8,13&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(13=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="O43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,14&gt;=Assumptions!$B$8,14&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(14=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(14&gt;=Assumptions!$B$8,14&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(14&gt;=Assumptions!$B$8,14&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(14&gt;=Assumptions!$B$8,14&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(14&gt;=Assumptions!$B$8,14&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(14&gt;=Assumptions!$B$8,14&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(14=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="P43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,15&gt;=Assumptions!$B$8,15&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(15=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(15&gt;=Assumptions!$B$8,15&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(15&gt;=Assumptions!$B$8,15&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(15&gt;=Assumptions!$B$8,15&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(15&gt;=Assumptions!$B$8,15&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(15&gt;=Assumptions!$B$8,15&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(15=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="Q43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,16&gt;=Assumptions!$B$8,16&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(16=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(16&gt;=Assumptions!$B$8,16&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(16&gt;=Assumptions!$B$8,16&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(16&gt;=Assumptions!$B$8,16&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(16&gt;=Assumptions!$B$8,16&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(16&gt;=Assumptions!$B$8,16&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(16=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="R43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,17&gt;=Assumptions!$B$8,17&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(17=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(17&gt;=Assumptions!$B$8,17&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(17&gt;=Assumptions!$B$8,17&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(17&gt;=Assumptions!$B$8,17&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(17&gt;=Assumptions!$B$8,17&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(17&gt;=Assumptions!$B$8,17&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(17=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="S43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,18&gt;=Assumptions!$B$8,18&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(18=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(18&gt;=Assumptions!$B$8,18&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(18&gt;=Assumptions!$B$8,18&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(18&gt;=Assumptions!$B$8,18&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(18&gt;=Assumptions!$B$8,18&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(18&gt;=Assumptions!$B$8,18&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(18=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="T43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,19&gt;=Assumptions!$B$8,19&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(19=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(19&gt;=Assumptions!$B$8,19&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(19&gt;=Assumptions!$B$8,19&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(19&gt;=Assumptions!$B$8,19&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(19&gt;=Assumptions!$B$8,19&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(19&gt;=Assumptions!$B$8,19&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(19=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="U43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,20&gt;=Assumptions!$B$8,20&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(20=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(20&gt;=Assumptions!$B$8,20&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(20&gt;=Assumptions!$B$8,20&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(20&gt;=Assumptions!$B$8,20&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(20&gt;=Assumptions!$B$8,20&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(20&gt;=Assumptions!$B$8,20&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(20=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="V43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,21&gt;=Assumptions!$B$8,21&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(21=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(21&gt;=Assumptions!$B$8,21&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(21&gt;=Assumptions!$B$8,21&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(21&gt;=Assumptions!$B$8,21&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(21&gt;=Assumptions!$B$8,21&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(21&gt;=Assumptions!$B$8,21&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(21=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="W43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,22&gt;=Assumptions!$B$8,22&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(22=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(22&gt;=Assumptions!$B$8,22&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(22&gt;=Assumptions!$B$8,22&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(22&gt;=Assumptions!$B$8,22&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(22&gt;=Assumptions!$B$8,22&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(22&gt;=Assumptions!$B$8,22&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(22=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="X43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,23&gt;=Assumptions!$B$8,23&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(23=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(23&gt;=Assumptions!$B$8,23&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(23&gt;=Assumptions!$B$8,23&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(23&gt;=Assumptions!$B$8,23&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(23&gt;=Assumptions!$B$8,23&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(23&gt;=Assumptions!$B$8,23&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(23=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="Y43" s="21" t="n">
-        <f aca="false">IF(AND(Assumptions!$B$59=1,24&gt;=Assumptions!$B$8,24&lt;Assumptions!$B$8+3),Assumptions!$B$60,0)+IF(24=Assumptions!$B$8,Assumptions!$B$61,0)</f>
+        <f aca="false">IF(AND(24&gt;=Assumptions!$B$8,24&lt;Assumptions!$B$8+Assumptions!$B$56),Assumptions!$B$55,0)+IF(AND(24&gt;=Assumptions!$B$8,24&lt;Assumptions!$B$8+Assumptions!$B$59),Assumptions!$B$58,0)+IF(AND(24&gt;=Assumptions!$B$8,24&lt;Assumptions!$B$8+Assumptions!$B$62),Assumptions!$B$61,0)+IF(AND(24&gt;=Assumptions!$B$8,24&lt;Assumptions!$B$8+Assumptions!$B$65),Assumptions!$B$64,0)+IF(AND(24&gt;=Assumptions!$B$8,24&lt;Assumptions!$B$8+Assumptions!$B$68),Assumptions!$B$67,0)+IF(24=Assumptions!$B$8,Assumptions!$B$72,0)</f>
         <v>0</v>
       </c>
       <c r="Z43" s="21" t="n">
         <f aca="false">SUM(B43:M43)</f>
-        <v>10500</v>
+        <v>15600</v>
       </c>
       <c r="AA43" s="21" t="n">
         <f aca="false">SUM(N43:Y43)</f>
@@ -6111,125 +6349,125 @@
       </c>
       <c r="AB43" s="21" t="n">
         <f aca="false">SUM(B43:Y43)</f>
-        <v>10500</v>
+        <v>15600</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="17" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="B44" s="21" t="n">
-        <f aca="false">IF(1&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
+        <f aca="false">IF(1&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(1&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(1&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(1&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(1&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="C44" s="21" t="n">
-        <f aca="false">IF(2&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
+        <f aca="false">IF(2&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(2&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(2&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(2&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(2&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="D44" s="21" t="n">
-        <f aca="false">IF(3&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
+        <f aca="false">IF(3&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(3&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(3&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(3&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(3&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="E44" s="21" t="n">
-        <f aca="false">IF(4&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
+        <f aca="false">IF(4&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(4&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(4&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(4&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(4&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="F44" s="21" t="n">
-        <f aca="false">IF(5&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
+        <f aca="false">IF(5&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(5&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(5&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(5&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(5&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="G44" s="21" t="n">
-        <f aca="false">IF(6&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
+        <f aca="false">IF(6&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(6&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(6&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(6&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(6&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="H44" s="21" t="n">
-        <f aca="false">IF(7&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>0</v>
+        <f aca="false">IF(7&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(7&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(7&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(7&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(7&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>838.637551144702</v>
       </c>
       <c r="I44" s="21" t="n">
-        <f aca="false">IF(8&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>0</v>
+        <f aca="false">IF(8&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(8&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(8&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(8&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(8&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>838.637551144702</v>
       </c>
       <c r="J44" s="21" t="n">
-        <f aca="false">IF(9&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>0</v>
+        <f aca="false">IF(9&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(9&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(9&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(9&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(9&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>838.637551144702</v>
       </c>
       <c r="K44" s="21" t="n">
-        <f aca="false">IF(10&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(10&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(10&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(10&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(10&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(10&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="L44" s="21" t="n">
-        <f aca="false">IF(11&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(11&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(11&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(11&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(11&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(11&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="M44" s="21" t="n">
-        <f aca="false">IF(12&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(12&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(12&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(12&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(12&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(12&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="N44" s="21" t="n">
-        <f aca="false">IF(13&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(13&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(13&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(13&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(13&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(13&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="O44" s="21" t="n">
-        <f aca="false">IF(14&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(14&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(14&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(14&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(14&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(14&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="P44" s="21" t="n">
-        <f aca="false">IF(15&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(15&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(15&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(15&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(15&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(15&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="Q44" s="21" t="n">
-        <f aca="false">IF(16&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(16&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(16&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(16&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(16&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(16&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="R44" s="21" t="n">
-        <f aca="false">IF(17&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(17&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(17&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(17&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(17&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(17&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="S44" s="21" t="n">
-        <f aca="false">IF(18&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(18&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(18&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(18&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(18&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(18&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="T44" s="21" t="n">
-        <f aca="false">IF(19&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(19&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(19&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(19&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(19&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(19&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="U44" s="21" t="n">
-        <f aca="false">IF(20&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(20&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(20&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(20&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(20&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(20&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="V44" s="21" t="n">
-        <f aca="false">IF(21&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(21&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(21&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(21&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(21&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(21&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="W44" s="21" t="n">
-        <f aca="false">IF(22&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(22&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(22&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(22&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(22&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(22&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="X44" s="21" t="n">
-        <f aca="false">IF(23&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(23&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(23&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(23&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(23&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(23&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="Y44" s="21" t="n">
-        <f aca="false">IF(24&gt;=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),-PMT(Assumptions!$B$57/12,Assumptions!$B$58,(Assumptions!$B$54+Assumptions!$B$55)*Assumptions!$B$56),0)</f>
-        <v>1660.66841810832</v>
+        <f aca="false">IF(24&gt;=Assumptions!$B$8+Assumptions!$B$56,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$54*Assumptions!$B$69),0)+IF(24&gt;=Assumptions!$B$8+Assumptions!$B$59,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$57*Assumptions!$B$69),0)+IF(24&gt;=Assumptions!$B$8+Assumptions!$B$62,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$60*Assumptions!$B$69),0)+IF(24&gt;=Assumptions!$B$8+Assumptions!$B$65,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$63*Assumptions!$B$69),0)+IF(24&gt;=Assumptions!$B$8+Assumptions!$B$68,-PMT(Assumptions!$B$70/12,Assumptions!$B$71,Assumptions!$B$66*Assumptions!$B$69),0)</f>
+        <v>2300.02575908002</v>
       </c>
       <c r="Z44" s="21" t="n">
         <f aca="false">SUM(B44:M44)</f>
-        <v>4982.00525432496</v>
+        <v>9415.98993067418</v>
       </c>
       <c r="AA44" s="21" t="n">
         <f aca="false">SUM(N44:Y44)</f>
-        <v>19928.0210172999</v>
+        <v>27600.3091089603</v>
       </c>
       <c r="AB44" s="21" t="n">
         <f aca="false">SUM(B44:Y44)</f>
-        <v>24910.0262716248</v>
+        <v>37016.2990396345</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="15" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="B45" s="22" t="n">
         <f aca="false">SUM(B33:B44)</f>
@@ -6257,92 +6495,92 @@
       </c>
       <c r="H45" s="22" t="n">
         <f aca="false">SUM(H33:H44)</f>
-        <v>19100</v>
+        <v>21638.6375511447</v>
       </c>
       <c r="I45" s="22" t="n">
         <f aca="false">SUM(I33:I44)</f>
-        <v>14600</v>
+        <v>17138.6375511447</v>
       </c>
       <c r="J45" s="22" t="n">
         <f aca="false">SUM(J33:J44)</f>
-        <v>14600</v>
+        <v>17138.6375511447</v>
       </c>
       <c r="K45" s="22" t="n">
         <f aca="false">SUM(K33:K44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="L45" s="22" t="n">
         <f aca="false">SUM(L33:L44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="M45" s="22" t="n">
         <f aca="false">SUM(M33:M44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="N45" s="22" t="n">
         <f aca="false">SUM(N33:N44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="O45" s="22" t="n">
         <f aca="false">SUM(O33:O44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="P45" s="22" t="n">
         <f aca="false">SUM(P33:P44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="Q45" s="22" t="n">
         <f aca="false">SUM(Q33:Q44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="R45" s="22" t="n">
         <f aca="false">SUM(R33:R44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="S45" s="22" t="n">
         <f aca="false">SUM(S33:S44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="T45" s="22" t="n">
         <f aca="false">SUM(T33:T44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="U45" s="22" t="n">
         <f aca="false">SUM(U33:U44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="V45" s="22" t="n">
         <f aca="false">SUM(V33:V44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="W45" s="22" t="n">
         <f aca="false">SUM(W33:W44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="X45" s="22" t="n">
         <f aca="false">SUM(X33:X44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="Y45" s="22" t="n">
         <f aca="false">SUM(Y33:Y44)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="Z45" s="23" t="n">
         <f aca="false">SUM(B45:M45)</f>
-        <v>160682.005254325</v>
+        <v>170215.989930674</v>
       </c>
       <c r="AA45" s="23" t="n">
         <f aca="false">SUM(N45:Y45)</f>
-        <v>171128.0210173</v>
+        <v>178800.30910896</v>
       </c>
       <c r="AB45" s="23" t="n">
         <f aca="false">SUM(B45:Y45)</f>
-        <v>331810.026271625</v>
+        <v>349016.299039634</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="15" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="B46" s="23" t="n">
         <f aca="false">B30-B45</f>
@@ -6370,92 +6608,92 @@
       </c>
       <c r="H46" s="23" t="n">
         <f aca="false">H30-H45</f>
-        <v>9539.26315171339</v>
+        <v>7000.62560056869</v>
       </c>
       <c r="I46" s="23" t="n">
         <f aca="false">I30-I45</f>
-        <v>16843.9523695909</v>
+        <v>14305.3148184462</v>
       </c>
       <c r="J46" s="23" t="n">
         <f aca="false">J30-J45</f>
-        <v>19655.8192149047</v>
+        <v>17117.18166376</v>
       </c>
       <c r="K46" s="23" t="n">
         <f aca="false">K30-K45</f>
-        <v>22814.147418697</v>
+        <v>22174.7900777253</v>
       </c>
       <c r="L46" s="23" t="n">
         <f aca="false">L30-L45</f>
-        <v>22944.270729785</v>
+        <v>22304.9133888133</v>
       </c>
       <c r="M46" s="23" t="n">
         <f aca="false">M30-M45</f>
-        <v>23073.5265521324</v>
+        <v>22434.1692111606</v>
       </c>
       <c r="N46" s="23" t="n">
         <f aca="false">N30-N45</f>
-        <v>23201.9206689974</v>
+        <v>22562.5633280257</v>
       </c>
       <c r="O46" s="23" t="n">
         <f aca="false">O30-O45</f>
-        <v>23329.4588250834</v>
+        <v>22690.1014841117</v>
       </c>
       <c r="P46" s="23" t="n">
         <f aca="false">P30-P45</f>
-        <v>23428.1779767954</v>
+        <v>22788.8206358237</v>
       </c>
       <c r="Q46" s="23" t="n">
         <f aca="false">Q30-Q45</f>
-        <v>23526.2390008294</v>
+        <v>22886.8816598577</v>
       </c>
       <c r="R46" s="23" t="n">
         <f aca="false">R30-R45</f>
-        <v>23623.6462847032</v>
+        <v>22984.2889437315</v>
       </c>
       <c r="S46" s="23" t="n">
         <f aca="false">S30-S45</f>
-        <v>23720.4041866844</v>
+        <v>23081.0468457127</v>
       </c>
       <c r="T46" s="23" t="n">
         <f aca="false">T30-T45</f>
-        <v>23816.5170359858</v>
+        <v>23177.1596950141</v>
       </c>
       <c r="U46" s="23" t="n">
         <f aca="false">U30-U45</f>
-        <v>23911.9891329585</v>
+        <v>23272.6317919868</v>
       </c>
       <c r="V46" s="23" t="n">
         <f aca="false">V30-V45</f>
-        <v>24006.8247492847</v>
+        <v>23367.467408313</v>
       </c>
       <c r="W46" s="23" t="n">
         <f aca="false">W30-W45</f>
-        <v>24101.0281281688</v>
+        <v>23461.6707871971</v>
       </c>
       <c r="X46" s="23" t="n">
         <f aca="false">X30-X45</f>
-        <v>24194.6034845269</v>
+        <v>23555.2461435552</v>
       </c>
       <c r="Y46" s="23" t="n">
         <f aca="false">Y30-Y45</f>
-        <v>24287.555005176</v>
+        <v>23648.1976642043</v>
       </c>
       <c r="Z46" s="23" t="n">
         <f aca="false">SUM(B46:M46)</f>
-        <v>139767.069179814</v>
+        <v>130233.084503465</v>
       </c>
       <c r="AA46" s="23" t="n">
         <f aca="false">SUM(N46:Y46)</f>
-        <v>285148.364479194</v>
+        <v>277476.076387534</v>
       </c>
       <c r="AB46" s="23" t="n">
         <f aca="false">SUM(B46:Y46)</f>
-        <v>424915.433659008</v>
+        <v>407709.160890998</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="17" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="B47" s="20" t="n">
         <f aca="false">IF(B24=0,0,B46/B24)</f>
@@ -6483,75 +6721,75 @@
       </c>
       <c r="H47" s="20" t="n">
         <f aca="false">IF(H24=0,0,H46/H24)</f>
-        <v>0.16065408613074</v>
+        <v>0.117899998177618</v>
       </c>
       <c r="I47" s="20" t="n">
         <f aca="false">IF(I24=0,0,I46/I24)</f>
-        <v>0.258580871133738</v>
+        <v>0.219608835647998</v>
       </c>
       <c r="J47" s="20" t="n">
         <f aca="false">IF(J24=0,0,J46/J24)</f>
-        <v>0.277184965371192</v>
+        <v>0.241385279079284</v>
       </c>
       <c r="K47" s="20" t="n">
         <f aca="false">IF(K24=0,0,K46/K24)</f>
-        <v>0.297467806527227</v>
+        <v>0.289131390429114</v>
       </c>
       <c r="L47" s="20" t="n">
         <f aca="false">IF(L24=0,0,L46/L24)</f>
-        <v>0.298460044457676</v>
+        <v>0.2901432571142</v>
       </c>
       <c r="M47" s="20" t="n">
         <f aca="false">IF(M24=0,0,M46/M24)</f>
-        <v>0.299441052278976</v>
+        <v>0.291143671532678</v>
       </c>
       <c r="N47" s="20" t="n">
         <f aca="false">IF(N24=0,0,N46/N24)</f>
-        <v>0.300410997994279</v>
+        <v>0.29213280501119</v>
       </c>
       <c r="O47" s="20" t="n">
         <f aca="false">IF(O24=0,0,O46/O24)</f>
-        <v>0.301370046328512</v>
+        <v>0.293110825533302</v>
       </c>
       <c r="P47" s="20" t="n">
         <f aca="false">IF(P24=0,0,P46/P24)</f>
-        <v>0.302109371629716</v>
+        <v>0.29386477639405</v>
       </c>
       <c r="Q47" s="20" t="n">
         <f aca="false">IF(Q24=0,0,Q46/Q24)</f>
-        <v>0.302841180355429</v>
+        <v>0.294611061984109</v>
       </c>
       <c r="R47" s="20" t="n">
         <f aca="false">IF(R24=0,0,R46/R24)</f>
-        <v>0.303565570431586</v>
+        <v>0.295349782166614</v>
       </c>
       <c r="S47" s="20" t="n">
         <f aca="false">IF(S24=0,0,S46/S24)</f>
-        <v>0.304282638137298</v>
+        <v>0.2960810351253</v>
       </c>
       <c r="T47" s="20" t="n">
         <f aca="false">IF(T24=0,0,T46/T24)</f>
-        <v>0.304992478139368</v>
+        <v>0.296804917399697</v>
       </c>
       <c r="U47" s="20" t="n">
         <f aca="false">IF(U24=0,0,U46/U24)</f>
-        <v>0.305695183525931</v>
+        <v>0.297521523919436</v>
       </c>
       <c r="V47" s="20" t="n">
         <f aca="false">IF(V24=0,0,V46/V24)</f>
-        <v>0.306390845839261</v>
+        <v>0.298230948037712</v>
       </c>
       <c r="W47" s="20" t="n">
         <f aca="false">IF(W24=0,0,W46/W24)</f>
-        <v>0.30707955510776</v>
+        <v>0.298933281563894</v>
       </c>
       <c r="X47" s="20" t="n">
         <f aca="false">IF(X24=0,0,X46/X24)</f>
-        <v>0.307761399877156</v>
+        <v>0.299628614795349</v>
       </c>
       <c r="Y47" s="20" t="n">
         <f aca="false">IF(Y24=0,0,Y46/Y24)</f>
-        <v>0.308436467240926</v>
+        <v>0.300317036548465</v>
       </c>
       <c r="Z47" s="2"/>
       <c r="AA47" s="2"/>
@@ -6559,7 +6797,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="B48" s="5"/>
       <c r="C48" s="5"/>
@@ -6591,7 +6829,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="17" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="B49" s="21" t="n">
         <f aca="false">B20*Assumptions!$B$29+B20*(1-Assumptions!$B$29)*Assumptions!$B$30+0+B23</f>
@@ -6704,7 +6942,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="17" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="B50" s="21" t="n">
         <f aca="false">B29+B45</f>
@@ -6732,192 +6970,192 @@
       </c>
       <c r="H50" s="21" t="n">
         <f aca="false">H29+H45</f>
-        <v>49838.3934112846</v>
+        <v>52377.0309624293</v>
       </c>
       <c r="I50" s="21" t="n">
         <f aca="false">I29+I45</f>
-        <v>48296.0260663205</v>
+        <v>50834.6636174652</v>
       </c>
       <c r="J50" s="21" t="n">
         <f aca="false">J29+J45</f>
-        <v>51256.4656147672</v>
+        <v>53795.1031659119</v>
       </c>
       <c r="K50" s="21" t="n">
         <f aca="false">K29+K45</f>
-        <v>53880.3617621104</v>
+        <v>54519.7191030821</v>
       </c>
       <c r="L50" s="21" t="n">
         <f aca="false">L29+L45</f>
-        <v>53931.2479731504</v>
+        <v>54570.6053141221</v>
       </c>
       <c r="M50" s="21" t="n">
         <f aca="false">M29+M45</f>
-        <v>53981.7949427835</v>
+        <v>54621.1522837552</v>
       </c>
       <c r="N50" s="21" t="n">
         <f aca="false">N29+N45</f>
-        <v>54032.0049326189</v>
+        <v>54671.3622735907</v>
       </c>
       <c r="O50" s="21" t="n">
         <f aca="false">O29+O45</f>
-        <v>54081.8801891889</v>
+        <v>54721.2375301606</v>
       </c>
       <c r="P50" s="21" t="n">
         <f aca="false">P29+P45</f>
-        <v>54120.4854440483</v>
+        <v>54759.84278502</v>
       </c>
       <c r="Q50" s="21" t="n">
         <f aca="false">Q29+Q45</f>
-        <v>54158.8333305421</v>
+        <v>54798.1906715138</v>
       </c>
       <c r="R50" s="21" t="n">
         <f aca="false">R29+R45</f>
-        <v>54196.9255644592</v>
+        <v>54836.2829054309</v>
       </c>
       <c r="S50" s="21" t="n">
         <f aca="false">S29+S45</f>
-        <v>54234.7638501502</v>
+        <v>54874.1211911219</v>
       </c>
       <c r="T50" s="21" t="n">
         <f aca="false">T29+T45</f>
-        <v>54272.3498806032</v>
+        <v>54911.7072215749</v>
       </c>
       <c r="U50" s="21" t="n">
         <f aca="false">U29+U45</f>
-        <v>54309.6853375199</v>
+        <v>54949.0426784916</v>
       </c>
       <c r="V50" s="21" t="n">
         <f aca="false">V29+V45</f>
-        <v>54346.7718913905</v>
+        <v>54986.1292323622</v>
       </c>
       <c r="W50" s="21" t="n">
         <f aca="false">W29+W45</f>
-        <v>54383.6112015686</v>
+        <v>55022.9685425403</v>
       </c>
       <c r="X50" s="21" t="n">
         <f aca="false">X29+X45</f>
-        <v>54420.2049163456</v>
+        <v>55059.5622573173</v>
       </c>
       <c r="Y50" s="21" t="n">
         <f aca="false">Y29+Y45</f>
-        <v>54456.554673024</v>
+        <v>55095.9120139957</v>
       </c>
       <c r="Z50" s="21" t="n">
         <f aca="false">SUM(B50:M50)</f>
-        <v>482634.403077731</v>
+        <v>492168.38775408</v>
       </c>
       <c r="AA50" s="21" t="n">
         <f aca="false">SUM(N50:Y50)</f>
-        <v>651014.071211459</v>
+        <v>658686.35930312</v>
       </c>
       <c r="AB50" s="21" t="n">
         <f aca="false">SUM(B50:Y50)</f>
-        <v>1133648.47428919</v>
+        <v>1150854.7470572</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="17" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="B51" s="21" t="n">
-        <f aca="false">IF(1=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(1=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(1=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(1=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(1=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(1=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="C51" s="21" t="n">
-        <f aca="false">IF(2=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(2=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(2=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(2=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(2=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(2=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="D51" s="21" t="n">
-        <f aca="false">IF(3=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(3=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(3=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(3=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(3=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(3=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="E51" s="21" t="n">
-        <f aca="false">IF(4=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(4=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(4=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(4=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(4=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(4=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="F51" s="21" t="n">
-        <f aca="false">IF(5=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(5=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(5=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(5=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(5=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(5=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="G51" s="21" t="n">
-        <f aca="false">IF(6=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(6=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(6=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(6=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(6=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(6=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="H51" s="21" t="n">
-        <f aca="false">IF(7=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
-        <v>0</v>
+        <f aca="false">IF(7=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(7=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(7=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(7=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(7=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
+        <v>10100</v>
       </c>
       <c r="I51" s="21" t="n">
-        <f aca="false">IF(8=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(8=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(8=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(8=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(8=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(8=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="J51" s="21" t="n">
-        <f aca="false">IF(9=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(9=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(9=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(9=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(9=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(9=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="K51" s="21" t="n">
-        <f aca="false">IF(10=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
-        <v>20000</v>
+        <f aca="false">IF(10=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(10=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(10=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(10=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(10=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
+        <v>17600</v>
       </c>
       <c r="L51" s="21" t="n">
-        <f aca="false">IF(11=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(11=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(11=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(11=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(11=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(11=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="M51" s="21" t="n">
-        <f aca="false">IF(12=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(12=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(12=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(12=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(12=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(12=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="N51" s="21" t="n">
-        <f aca="false">IF(13=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(13=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(13=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(13=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(13=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(13=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="O51" s="21" t="n">
-        <f aca="false">IF(14=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(14=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(14=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(14=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(14=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(14=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="P51" s="21" t="n">
-        <f aca="false">IF(15=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(15=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(15=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(15=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(15=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(15=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="Q51" s="21" t="n">
-        <f aca="false">IF(16=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(16=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(16=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(16=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(16=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(16=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="R51" s="21" t="n">
-        <f aca="false">IF(17=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(17=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(17=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(17=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(17=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(17=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="S51" s="21" t="n">
-        <f aca="false">IF(18=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(18=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(18=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(18=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(18=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(18=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="T51" s="21" t="n">
-        <f aca="false">IF(19=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(19=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(19=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(19=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(19=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(19=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="U51" s="21" t="n">
-        <f aca="false">IF(20=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(20=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(20=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(20=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(20=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(20=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="V51" s="21" t="n">
-        <f aca="false">IF(21=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(21=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(21=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(21=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(21=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(21=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="W51" s="21" t="n">
-        <f aca="false">IF(22=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(22=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(22=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(22=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(22=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(22=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="X51" s="21" t="n">
-        <f aca="false">IF(23=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(23=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(23=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(23=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(23=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(23=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="Y51" s="21" t="n">
-        <f aca="false">IF(24=Assumptions!$B$8+IF(Assumptions!$B$59=1,3,0),(Assumptions!$B$54+Assumptions!$B$55)*(1-Assumptions!$B$56),0)</f>
+        <f aca="false">IF(24=Assumptions!$B$8+Assumptions!$B$56,Assumptions!$B$54*(1-Assumptions!$B$69),0)+IF(24=Assumptions!$B$8+Assumptions!$B$59,Assumptions!$B$57*(1-Assumptions!$B$69),0)+IF(24=Assumptions!$B$8+Assumptions!$B$62,Assumptions!$B$60*(1-Assumptions!$B$69),0)+IF(24=Assumptions!$B$8+Assumptions!$B$65,Assumptions!$B$63*(1-Assumptions!$B$69),0)+IF(24=Assumptions!$B$8+Assumptions!$B$68,Assumptions!$B$66*(1-Assumptions!$B$69),0)</f>
         <v>0</v>
       </c>
       <c r="Z51" s="21" t="n">
         <f aca="false">SUM(B51:M51)</f>
-        <v>20000</v>
+        <v>27700</v>
       </c>
       <c r="AA51" s="21" t="n">
         <f aca="false">SUM(N51:Y51)</f>
@@ -6925,12 +7163,12 @@
       </c>
       <c r="AB51" s="21" t="n">
         <f aca="false">SUM(B51:Y51)</f>
-        <v>20000</v>
+        <v>27700</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="15" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="B52" s="22" t="n">
         <f aca="false">B49-B50-B51</f>
@@ -6958,92 +7196,92 @@
       </c>
       <c r="H52" s="22" t="n">
         <f aca="false">H49-H50-H51</f>
-        <v>8069.26315171339</v>
+        <v>-4569.37439943131</v>
       </c>
       <c r="I52" s="22" t="n">
         <f aca="false">I49-I50-I51</f>
-        <v>16451.9523695909</v>
+        <v>13913.3148184462</v>
       </c>
       <c r="J52" s="22" t="n">
         <f aca="false">J49-J50-J51</f>
-        <v>19263.8192149047</v>
+        <v>16725.18166376</v>
       </c>
       <c r="K52" s="22" t="n">
         <f aca="false">K49-K50-K51</f>
-        <v>2422.14741869702</v>
+        <v>4182.79007772531</v>
       </c>
       <c r="L52" s="22" t="n">
         <f aca="false">L49-L50-L51</f>
-        <v>22944.270729785</v>
+        <v>22304.9133888133</v>
       </c>
       <c r="M52" s="22" t="n">
         <f aca="false">M49-M50-M51</f>
-        <v>23073.5265521324</v>
+        <v>22434.1692111606</v>
       </c>
       <c r="N52" s="22" t="n">
         <f aca="false">N49-N50-N51</f>
-        <v>23201.9206689974</v>
+        <v>22562.5633280257</v>
       </c>
       <c r="O52" s="22" t="n">
         <f aca="false">O49-O50-O51</f>
-        <v>23329.4588250834</v>
+        <v>22690.1014841117</v>
       </c>
       <c r="P52" s="22" t="n">
         <f aca="false">P49-P50-P51</f>
-        <v>23428.1779767954</v>
+        <v>22788.8206358237</v>
       </c>
       <c r="Q52" s="22" t="n">
         <f aca="false">Q49-Q50-Q51</f>
-        <v>23526.2390008294</v>
+        <v>22886.8816598577</v>
       </c>
       <c r="R52" s="22" t="n">
         <f aca="false">R49-R50-R51</f>
-        <v>23623.6462847032</v>
+        <v>22984.2889437315</v>
       </c>
       <c r="S52" s="22" t="n">
         <f aca="false">S49-S50-S51</f>
-        <v>23720.4041866844</v>
+        <v>23081.0468457127</v>
       </c>
       <c r="T52" s="22" t="n">
         <f aca="false">T49-T50-T51</f>
-        <v>23816.5170359858</v>
+        <v>23177.1596950141</v>
       </c>
       <c r="U52" s="22" t="n">
         <f aca="false">U49-U50-U51</f>
-        <v>23911.9891329585</v>
+        <v>23272.6317919868</v>
       </c>
       <c r="V52" s="22" t="n">
         <f aca="false">V49-V50-V51</f>
-        <v>24006.8247492847</v>
+        <v>23367.467408313</v>
       </c>
       <c r="W52" s="22" t="n">
         <f aca="false">W49-W50-W51</f>
-        <v>24101.0281281688</v>
+        <v>23461.6707871971</v>
       </c>
       <c r="X52" s="22" t="n">
         <f aca="false">X49-X50-X51</f>
-        <v>24194.6034845269</v>
+        <v>23555.2461435552</v>
       </c>
       <c r="Y52" s="22" t="n">
         <f aca="false">Y49-Y50-Y51</f>
-        <v>24287.555005176</v>
+        <v>23648.1976642043</v>
       </c>
       <c r="Z52" s="23" t="n">
         <f aca="false">SUM(B52:M52)</f>
-        <v>114475.069179814</v>
+        <v>97241.0845034648</v>
       </c>
       <c r="AA52" s="23" t="n">
         <f aca="false">SUM(N52:Y52)</f>
-        <v>285148.364479194</v>
+        <v>277476.076387534</v>
       </c>
       <c r="AB52" s="23" t="n">
         <f aca="false">SUM(B52:Y52)</f>
-        <v>399623.433659008</v>
+        <v>374717.160890998</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="15" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="B53" s="23" t="n">
         <f aca="false">Assumptions!$B$32+B52</f>
@@ -7071,75 +7309,75 @@
       </c>
       <c r="H53" s="23" t="n">
         <f aca="false">G53+H52</f>
-        <v>55319.3528947041</v>
+        <v>42680.7153435594</v>
       </c>
       <c r="I53" s="23" t="n">
         <f aca="false">H53+I52</f>
-        <v>71771.305264295</v>
+        <v>56594.0301620056</v>
       </c>
       <c r="J53" s="23" t="n">
         <f aca="false">I53+J52</f>
-        <v>91035.1244791997</v>
+        <v>73319.2118257656</v>
       </c>
       <c r="K53" s="23" t="n">
         <f aca="false">J53+K52</f>
-        <v>93457.2718978967</v>
+        <v>77502.0019034909</v>
       </c>
       <c r="L53" s="23" t="n">
         <f aca="false">K53+L52</f>
-        <v>116401.542627682</v>
+        <v>99806.9152923042</v>
       </c>
       <c r="M53" s="23" t="n">
         <f aca="false">L53+M52</f>
-        <v>139475.069179814</v>
+        <v>122241.084503465</v>
       </c>
       <c r="N53" s="23" t="n">
         <f aca="false">M53+N52</f>
-        <v>162676.989848811</v>
+        <v>144803.647831491</v>
       </c>
       <c r="O53" s="23" t="n">
         <f aca="false">N53+O52</f>
-        <v>186006.448673895</v>
+        <v>167493.749315602</v>
       </c>
       <c r="P53" s="23" t="n">
         <f aca="false">O53+P52</f>
-        <v>209434.62665069</v>
+        <v>190282.569951426</v>
       </c>
       <c r="Q53" s="23" t="n">
         <f aca="false">P53+Q52</f>
-        <v>232960.86565152</v>
+        <v>213169.451611284</v>
       </c>
       <c r="R53" s="23" t="n">
         <f aca="false">Q53+R52</f>
-        <v>256584.511936223</v>
+        <v>236153.740555015</v>
       </c>
       <c r="S53" s="23" t="n">
         <f aca="false">R53+S52</f>
-        <v>280304.916122907</v>
+        <v>259234.787400728</v>
       </c>
       <c r="T53" s="23" t="n">
         <f aca="false">S53+T52</f>
-        <v>304121.433158893</v>
+        <v>282411.947095742</v>
       </c>
       <c r="U53" s="23" t="n">
         <f aca="false">T53+U52</f>
-        <v>328033.422291852</v>
+        <v>305684.578887729</v>
       </c>
       <c r="V53" s="23" t="n">
         <f aca="false">U53+V52</f>
-        <v>352040.247041136</v>
+        <v>329052.046296042</v>
       </c>
       <c r="W53" s="23" t="n">
         <f aca="false">V53+W52</f>
-        <v>376141.275169305</v>
+        <v>352513.717083239</v>
       </c>
       <c r="X53" s="23" t="n">
         <f aca="false">W53+X52</f>
-        <v>400335.878653832</v>
+        <v>376068.963226794</v>
       </c>
       <c r="Y53" s="23" t="n">
         <f aca="false">X53+Y52</f>
-        <v>424623.433659008</v>
+        <v>399717.160890998</v>
       </c>
       <c r="Z53" s="2"/>
       <c r="AA53" s="2"/>
@@ -7147,7 +7385,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="B54" s="5"/>
       <c r="C54" s="5"/>
@@ -7179,7 +7417,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="17" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="B55" s="21" t="n">
         <f aca="false">IF(B8=0,0,B20/IF(B7&gt;0,2,1))</f>
@@ -7283,7 +7521,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="17" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="B56" s="21" t="n">
         <f aca="false">IF(B13=0,0,(B40+B41+B42)/B13)</f>
@@ -7387,7 +7625,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="17" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="B57" s="21" t="n">
         <f aca="false">IF(B14=0,0,(B40+B41+B42)/B14)</f>
@@ -7491,7 +7729,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="17" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="B58" s="20" t="n">
         <f aca="false">IF(B24=0,0,B23/B24)</f>
@@ -7595,7 +7833,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="17" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="B59" s="18" t="n">
         <f aca="false">B45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
@@ -7623,75 +7861,75 @@
       </c>
       <c r="H59" s="18" t="n">
         <f aca="false">H45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>947.420634920635</v>
+        <v>1073.34511662424</v>
       </c>
       <c r="I59" s="18" t="n">
         <f aca="false">I45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>724.206349206349</v>
+        <v>850.130830909956</v>
       </c>
       <c r="J59" s="18" t="n">
         <f aca="false">J45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>724.206349206349</v>
+        <v>850.130830909956</v>
       </c>
       <c r="K59" s="18" t="n">
         <f aca="false">K45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="L59" s="18" t="n">
         <f aca="false">L45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="M59" s="18" t="n">
         <f aca="false">M45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="N59" s="18" t="n">
         <f aca="false">N45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="O59" s="18" t="n">
         <f aca="false">O45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="P59" s="18" t="n">
         <f aca="false">P45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="Q59" s="18" t="n">
         <f aca="false">Q45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="R59" s="18" t="n">
         <f aca="false">R45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="S59" s="18" t="n">
         <f aca="false">S45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="T59" s="18" t="n">
         <f aca="false">T45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="U59" s="18" t="n">
         <f aca="false">U45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="V59" s="18" t="n">
         <f aca="false">V45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="W59" s="18" t="n">
         <f aca="false">W45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="X59" s="18" t="n">
         <f aca="false">X45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="Y59" s="18" t="n">
         <f aca="false">Y45/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
-        <v>707.374425501405</v>
+        <v>739.088579319446</v>
       </c>
       <c r="Z59" s="2"/>
       <c r="AA59" s="2"/>
@@ -7723,21 +7961,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="B3" s="24" t="n">
         <f aca="false">Assumptions!$B$11</f>
@@ -7747,7 +7985,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
       <c r="B4" s="25" t="n">
         <f aca="false">B3*Assumptions!$B$5</f>
@@ -7757,7 +7995,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="B5" s="25" t="n">
         <f aca="false">B4*Assumptions!$B$14</f>
@@ -7767,7 +8005,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="B6" s="25" t="n">
         <f aca="false">B4*Assumptions!$B$15</f>
@@ -7777,7 +8015,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="B7" s="21" t="n">
         <f aca="false">B4-B5-B6</f>
@@ -7787,7 +8025,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="B8" s="20" t="n">
         <f aca="false">B7/B4</f>
@@ -7797,7 +8035,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
       <c r="B9" s="26" t="n">
         <f aca="false">B3/(Assumptions!$B$7/21)</f>
@@ -7807,14 +8045,14 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>178</v>
+        <v>194</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>179</v>
+        <v>195</v>
       </c>
       <c r="B11" s="24" t="n">
         <f aca="false">Assumptions!$B$7</f>
@@ -7824,7 +8062,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="B12" s="25" t="n">
         <f aca="false">B11*Assumptions!$B$5</f>
@@ -7834,7 +8072,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>180</v>
+        <v>196</v>
       </c>
       <c r="B13" s="25" t="n">
         <f aca="false">Assumptions!$B$18*Assumptions!$B$19*Assumptions!$B$16</f>
@@ -7844,7 +8082,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
       <c r="B14" s="25" t="n">
         <f aca="false">B13*(1+Assumptions!$B$17)</f>
@@ -7854,19 +8092,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="B15" s="20" t="n">
         <f aca="false">B14/B12</f>
         <v>0.352178571428572</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="B16" s="25" t="n">
         <f aca="false">B12*(1-Assumptions!$B$14-Assumptions!$B$15)</f>
@@ -7876,14 +8114,14 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="B18" s="25" t="n">
         <f aca="false">Assumptions!$B$21</f>
@@ -7893,7 +8131,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="B19" s="25" t="n">
         <f aca="false">Assumptions!$B$27</f>
@@ -7903,7 +8141,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
       <c r="B20" s="21" t="n">
         <f aca="false">B18-B19</f>
@@ -7913,7 +8151,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="B21" s="20" t="n">
         <f aca="false">B20/B18</f>
@@ -7923,7 +8161,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="B22" s="24" t="n">
         <f aca="false">5/Assumptions!$B$22</f>
@@ -7933,7 +8171,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>191</v>
+        <v>207</v>
       </c>
       <c r="B23" s="21" t="n">
         <f aca="false">B20*B22</f>
@@ -7943,26 +8181,26 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>192</v>
+        <v>208</v>
       </c>
       <c r="B24" s="21" t="n">
         <f aca="false">0.25*B4*(1-0.52)</f>
         <v>504</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>193</v>
+        <v>209</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
       <c r="B26" s="25" t="n">
         <f aca="false">'Proforma 24 mo'!D45</f>
@@ -7972,7 +8210,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
       <c r="B27" s="24" t="n">
         <f aca="false">B26/(Assumptions!$B$5*(1-Assumptions!$B$14-Assumptions!$B$15))</f>
@@ -7982,7 +8220,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
       <c r="B28" s="27" t="n">
         <f aca="false">B27/Assumptions!$B$7</f>
@@ -8015,7 +8253,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -8023,7 +8261,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>199</v>
+        <v>215</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -8038,18 +8276,18 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="28"/>
       <c r="B4" s="28" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="D4" s="28" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>700</v>
@@ -8063,7 +8301,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>1</v>
@@ -8077,7 +8315,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>38</v>
@@ -8091,7 +8329,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>40</v>
@@ -8105,7 +8343,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
       <c r="B9" s="21" t="n">
         <f aca="false">B5*B6*B7</f>
@@ -8122,7 +8360,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>208</v>
+        <v>224</v>
       </c>
       <c r="B10" s="21" t="n">
         <f aca="false">B8/12/Assumptions!$B$22*Assumptions!$B$21</f>
@@ -8139,7 +8377,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="B11" s="21" t="n">
         <f aca="false">B9+B10</f>
@@ -8156,7 +8394,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="B12" s="23" t="n">
         <f aca="false">B9*(1-Assumptions!$B$14-Assumptions!$B$15)+B10*(1-Assumptions!$B$27/Assumptions!$B$21)</f>
@@ -8173,7 +8411,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
       <c r="B13" s="21" t="n">
         <f aca="false">IF(B6=1,'Proforma 24 mo'!D45,'Proforma 24 mo'!Y45)</f>
@@ -8181,16 +8419,16 @@
       </c>
       <c r="C13" s="21" t="n">
         <f aca="false">IF(C6=1,'Proforma 24 mo'!D45,'Proforma 24 mo'!Y45)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
       <c r="D13" s="21" t="n">
         <f aca="false">IF(D6=1,'Proforma 24 mo'!D45,'Proforma 24 mo'!Y45)</f>
-        <v>14260.6684181083</v>
+        <v>14900.02575908</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="B14" s="23" t="n">
         <f aca="false">B12-B13</f>
@@ -8198,16 +8436,16 @@
       </c>
       <c r="C14" s="23" t="n">
         <f aca="false">C12-C13</f>
-        <v>23369.8315818917</v>
+        <v>22730.47424092</v>
       </c>
       <c r="D14" s="23" t="n">
         <f aca="false">D12-D13</f>
-        <v>31987.664915225</v>
+        <v>31348.3075742533</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="B15" s="23" t="n">
         <f aca="false">B14*12</f>
@@ -8215,16 +8453,16 @@
       </c>
       <c r="C15" s="23" t="n">
         <f aca="false">C14*12</f>
-        <v>280437.9789827</v>
+        <v>272765.69089104</v>
       </c>
       <c r="D15" s="23" t="n">
         <f aca="false">D14*12</f>
-        <v>383851.9789827</v>
+        <v>376179.69089104</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
       <c r="B16" s="20" t="n">
         <f aca="false">IF(B11=0,0,B14/B11)</f>
@@ -8232,16 +8470,16 @@
       </c>
       <c r="C16" s="20" t="n">
         <f aca="false">IF(C11=0,0,C14/C11)</f>
-        <v>0.301672721875518</v>
+        <v>0.293419488700681</v>
       </c>
       <c r="D16" s="20" t="n">
         <f aca="false">IF(D11=0,0,D14/D11)</f>
-        <v>0.337049311577104</v>
+        <v>0.33031249748963</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="B17" s="18" t="n">
         <f aca="false">B5*B6/Assumptions!$B$11/0.3</f>
@@ -8264,7 +8502,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="29" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -8272,7 +8510,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -8280,7 +8518,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -8288,7 +8526,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -8310,6 +8548,435 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="2" style="0" width="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="30" t="s">
+        <v>238</v>
+      </c>
+      <c r="B4" s="30" t="s">
+        <v>239</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>240</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>241</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>242</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>243</v>
+      </c>
+      <c r="G4" s="30" t="s">
+        <v>244</v>
+      </c>
+      <c r="H4" s="30" t="s">
+        <v>245</v>
+      </c>
+      <c r="I4" s="30" t="s">
+        <v>246</v>
+      </c>
+      <c r="J4" s="30" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B5" s="25" t="n">
+        <f aca="false">Assumptions!$B$54</f>
+        <v>50000</v>
+      </c>
+      <c r="C5" s="25" t="n">
+        <f aca="false">Assumptions!$B$55</f>
+        <v>2000</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <f aca="false">Assumptions!$B$56</f>
+        <v>3</v>
+      </c>
+      <c r="E5" s="21" t="n">
+        <f aca="false">C5*D5</f>
+        <v>6000</v>
+      </c>
+      <c r="F5" s="18" t="n">
+        <f aca="false">Assumptions!$B$8+D5</f>
+        <v>10</v>
+      </c>
+      <c r="G5" s="21" t="n">
+        <f aca="false">B5*(1-Assumptions!$B$69)</f>
+        <v>10000</v>
+      </c>
+      <c r="H5" s="21" t="n">
+        <f aca="false">-PMT(Assumptions!$B$70/12,Assumptions!$B$71,B5*Assumptions!$B$69)</f>
+        <v>830.33420905416</v>
+      </c>
+      <c r="I5" s="18" t="n">
+        <f aca="false">F5+Assumptions!$B$71</f>
+        <v>70</v>
+      </c>
+      <c r="J5" s="18" t="n">
+        <f aca="false">IF(C5=0,"n/a",B5/C5)</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B6" s="25" t="n">
+        <f aca="false">Assumptions!$B$57</f>
+        <v>38000</v>
+      </c>
+      <c r="C6" s="25" t="n">
+        <f aca="false">Assumptions!$B$58</f>
+        <v>1700</v>
+      </c>
+      <c r="D6" s="24" t="n">
+        <f aca="false">Assumptions!$B$59</f>
+        <v>3</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <f aca="false">C6*D6</f>
+        <v>5100</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <f aca="false">Assumptions!$B$8+D6</f>
+        <v>10</v>
+      </c>
+      <c r="G6" s="21" t="n">
+        <f aca="false">B6*(1-Assumptions!$B$69)</f>
+        <v>7600</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <f aca="false">-PMT(Assumptions!$B$70/12,Assumptions!$B$71,B6*Assumptions!$B$69)</f>
+        <v>631.053998881162</v>
+      </c>
+      <c r="I6" s="18" t="n">
+        <f aca="false">F6+Assumptions!$B$71</f>
+        <v>70</v>
+      </c>
+      <c r="J6" s="18" t="n">
+        <f aca="false">IF(C6=0,"n/a",B6/C6)</f>
+        <v>22.3529411764706</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B7" s="25" t="n">
+        <f aca="false">Assumptions!$B$60</f>
+        <v>9500</v>
+      </c>
+      <c r="C7" s="25" t="n">
+        <f aca="false">Assumptions!$B$61</f>
+        <v>600</v>
+      </c>
+      <c r="D7" s="24" t="n">
+        <f aca="false">Assumptions!$B$62</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <f aca="false">C7*D7</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <f aca="false">Assumptions!$B$8+D7</f>
+        <v>7</v>
+      </c>
+      <c r="G7" s="21" t="n">
+        <f aca="false">B7*(1-Assumptions!$B$69)</f>
+        <v>1900</v>
+      </c>
+      <c r="H7" s="21" t="n">
+        <f aca="false">-PMT(Assumptions!$B$70/12,Assumptions!$B$71,B7*Assumptions!$B$69)</f>
+        <v>157.76349972029</v>
+      </c>
+      <c r="I7" s="18" t="n">
+        <f aca="false">F7+Assumptions!$B$71</f>
+        <v>67</v>
+      </c>
+      <c r="J7" s="18" t="n">
+        <f aca="false">IF(C7=0,"n/a",B7/C7)</f>
+        <v>15.8333333333333</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B8" s="25" t="n">
+        <f aca="false">Assumptions!$B$63</f>
+        <v>35000</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <f aca="false">Assumptions!$B$64</f>
+        <v>0</v>
+      </c>
+      <c r="D8" s="24" t="n">
+        <f aca="false">Assumptions!$B$65</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <f aca="false">C8*D8</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <f aca="false">Assumptions!$B$8+D8</f>
+        <v>7</v>
+      </c>
+      <c r="G8" s="21" t="n">
+        <f aca="false">B8*(1-Assumptions!$B$69)</f>
+        <v>7000</v>
+      </c>
+      <c r="H8" s="21" t="n">
+        <f aca="false">-PMT(Assumptions!$B$70/12,Assumptions!$B$71,B8*Assumptions!$B$69)</f>
+        <v>581.233946337912</v>
+      </c>
+      <c r="I8" s="18" t="n">
+        <f aca="false">F8+Assumptions!$B$71</f>
+        <v>67</v>
+      </c>
+      <c r="J8" s="18" t="str">
+        <f aca="false">IF(C8=0,"n/a",B8/C8)</f>
+        <v>n/a</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B9" s="25" t="n">
+        <f aca="false">Assumptions!$B$66</f>
+        <v>6000</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <f aca="false">Assumptions!$B$67</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <f aca="false">Assumptions!$B$68</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <f aca="false">C9*D9</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <f aca="false">Assumptions!$B$8+D9</f>
+        <v>7</v>
+      </c>
+      <c r="G9" s="21" t="n">
+        <f aca="false">B9*(1-Assumptions!$B$69)</f>
+        <v>1200</v>
+      </c>
+      <c r="H9" s="21" t="n">
+        <f aca="false">-PMT(Assumptions!$B$70/12,Assumptions!$B$71,B9*Assumptions!$B$69)</f>
+        <v>99.6401050864993</v>
+      </c>
+      <c r="I9" s="18" t="n">
+        <f aca="false">F9+Assumptions!$B$71</f>
+        <v>67</v>
+      </c>
+      <c r="J9" s="18" t="str">
+        <f aca="false">IF(C9=0,"n/a",B9/C9)</f>
+        <v>n/a</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="15" t="s">
+        <v>253</v>
+      </c>
+      <c r="B10" s="23" t="n">
+        <f aca="false">SUM(B5:B9)</f>
+        <v>138500</v>
+      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="23" t="n">
+        <f aca="false">SUM(E5:E9)</f>
+        <v>11100</v>
+      </c>
+      <c r="F10" s="2"/>
+      <c r="G10" s="23" t="n">
+        <f aca="false">SUM(G5:G9)</f>
+        <v>27700</v>
+      </c>
+      <c r="H10" s="23" t="n">
+        <f aca="false">SUM(H5:H9)</f>
+        <v>2300.02575908002</v>
+      </c>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="29" t="s">
+        <v>254</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="31" t="s">
+        <v>255</v>
+      </c>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
+      <c r="J13" s="31"/>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="31" t="s">
+        <v>256</v>
+      </c>
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="31"/>
+      <c r="J14" s="31"/>
+    </row>
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="31" t="s">
+        <v>257</v>
+      </c>
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="31"/>
+      <c r="I15" s="31"/>
+      <c r="J15" s="31"/>
+    </row>
+    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+    </row>
+    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="31" t="s">
+        <v>259</v>
+      </c>
+      <c r="B17" s="31"/>
+      <c r="C17" s="31"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="31"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="31"/>
+      <c r="J17" s="31"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="A14:J14"/>
+    <mergeCell ref="A15:J15"/>
+    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A17:J17"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -8319,7 +8986,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>220</v>
+        <v>260</v>
       </c>
       <c r="B1" s="2"/>
     </row>
@@ -8328,99 +8995,99 @@
       <c r="B2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="30" t="s">
-        <v>221</v>
-      </c>
-      <c r="B3" s="31" t="s">
-        <v>222</v>
+      <c r="A3" s="32" t="s">
+        <v>261</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="30" t="s">
-        <v>223</v>
-      </c>
-      <c r="B4" s="31" t="s">
-        <v>224</v>
+      <c r="A4" s="32" t="s">
+        <v>263</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="30" t="s">
-        <v>225</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>226</v>
+      <c r="A5" s="32" t="s">
+        <v>265</v>
+      </c>
+      <c r="B5" s="33" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="30" t="s">
-        <v>227</v>
-      </c>
-      <c r="B6" s="31" t="s">
-        <v>228</v>
+      <c r="A6" s="32" t="s">
+        <v>267</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="30" t="s">
-        <v>229</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>230</v>
+      <c r="A7" s="32" t="s">
+        <v>269</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="30" t="s">
-        <v>231</v>
-      </c>
-      <c r="B8" s="31" t="s">
-        <v>232</v>
+      <c r="A8" s="32" t="s">
+        <v>271</v>
+      </c>
+      <c r="B8" s="33" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="30" t="s">
-        <v>233</v>
-      </c>
-      <c r="B9" s="31" t="s">
-        <v>234</v>
+      <c r="A9" s="32" t="s">
+        <v>273</v>
+      </c>
+      <c r="B9" s="33" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="30" t="s">
-        <v>235</v>
-      </c>
-      <c r="B10" s="31" t="s">
-        <v>236</v>
+      <c r="A10" s="32" t="s">
+        <v>275</v>
+      </c>
+      <c r="B10" s="33" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="30" t="s">
-        <v>237</v>
-      </c>
-      <c r="B11" s="31" t="s">
-        <v>238</v>
+      <c r="A11" s="32" t="s">
+        <v>277</v>
+      </c>
+      <c r="B11" s="33" t="s">
+        <v>278</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="30" t="s">
-        <v>239</v>
-      </c>
-      <c r="B12" s="31" t="s">
-        <v>240</v>
+      <c r="A12" s="32" t="s">
+        <v>279</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="30" t="s">
-        <v>241</v>
-      </c>
-      <c r="B13" s="31" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="30" t="s">
-        <v>243</v>
-      </c>
-      <c r="B14" s="31" t="s">
-        <v>244</v>
+      <c r="A13" s="32" t="s">
+        <v>281</v>
+      </c>
+      <c r="B13" s="33" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="32" t="s">
+        <v>283</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: five-year plan tab, year-by-year build, growth-lead proposal and valuation pages
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LoK8Mi2K1W9PhhoHM3MdEb
</commit_message>
<xml_diff>
--- a/docs/Scag-Scapes-Proforma.xlsx
+++ b/docs/Scag-Scapes-Proforma.xlsx
@@ -13,7 +13,8 @@
     <sheet name="Unit economics" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Scenarios" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Equipment plan" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Sources &amp; notes" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="5-year plan" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Sources &amp; notes" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="395">
   <si>
     <t xml:space="preserve">Scag Scapes LLC - Growth Proforma - Assumptions</t>
   </si>
@@ -915,6 +916,222 @@
     <t xml:space="preserve">Time to full ownership of Crew 2's set: trailer, truck and tools on day one; mini-ex and skid steer bought in month start+3; all loans paid off 60 months after that (month 70 in the base case). Equity builds from the first payment; the machines outlast the loans.</t>
   </si>
   <si>
+    <t xml:space="preserve">Five-year plan - annual, safe-scaling (Year 1-2 pull from the 24-month proforma; Years 3-5 from the blue inputs below)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue = input. Every year is gated: the next crew is added only when the previous one has run at target for 3 months, backlog &gt; 4 weeks, and cash &gt; 2 months of overhead.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Today (run rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAPACITY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crews at year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew 3 in year 3, Crew 4 in year 4, then consolidate. Change to test a slower or faster path.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average crews running during the year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew 3 starts mid-year 3; Crew 4 mid-year 4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LF per crew per year at target x utilization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Today = 400 LF x 12. Years 3-5: 900 LF x 12 x 95% utilization.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total LF installed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average $/LF (3% a year after year 2 - reviews and the map justify it)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drainage + other install revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Years 1-2 include other-work days; years 3-5 crews are full on drainage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drain Check active plans at year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40% attach on installs plus past customers; ~8%/yr churn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drain Check revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew labor (crews x fixed crew cost; wages +3%/yr from year 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change the wage on Assumptions and every year moves.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drain Check visit costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OVERHEAD - the layers that let the company handle the volume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charlie's pay rises with the company.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Office admin / bookkeeper (part-time year 2, full-time year 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answers the phone the software cannot, books, AP/AR, reviews, scheduling. Hire when two crews are running.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operations manager (runs crews, purchasing, quality)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hired in month 4 of year 3 (about $65K/yr), before Crew 3 starts, so Charlie is not the bottleneck at three crews. Usually the best crew lead, promoted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimator / sales (runs Moasure surveys and quotes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At four crews Charlie cannot run 40+ estimates a month alone. Base + commission.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew-lead bonus pool (LF/day and callbacks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$500/quarter per lead when the crew beats 43 LF/day with no callbacks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insurance - GL, auto, equipment, WC excess (per crew)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Today's premium plus about $9K per additional crew (auto, equipment, WC); get quotes before each hire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Truck + equipment loan payments (existing + one set per crew)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each new crew carries its own set (Equipment plan tab); rent-first 3 months before each purchase.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yard / shop (Cottondale: 2,500 sq ft yr 2, 3,000 sq ft yr 3, 4,000 sq ft yr 4+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introductory $0.85 then $1.05/sq ft; more footage as crews and bins are added.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software, phones, hosting, payment fees (+ per crew)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bookkeeping / CPA / payroll service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QuickBooks Online + payroll service + monthly close; CPA quarterly. Grows with headcount.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marketing (Google LSA, Meta, content) - ~5% of revenue from year 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Falls as a % of revenue as reviews, referrals and the plan book compound.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shop, tools, uniforms, training, misc (+ per crew)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew hiring, training and rent-first equipment months (per new crew)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROWTH &amp; OPERATIONS LEAD (Ned) - proposed, for discussion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base ($/yr) - fractional, about 25 hours a week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For scale: Baton Rouge general/operations managers average $129,840 full-time (BLS OEWS). Set to 0 to see the plan without it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth share - % of operating profit above the baseline year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid only on profit above what the business makes today; nothing on the baseline.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseline operating profit (today's run rate after owner draw, floored at 0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Today's column, computed below. The share is earned only on profit the growth creates.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth lead cost (base + share)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share is computed on operating profit before the share itself.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL OVERHEAD (excl. growth lead)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operating profit before growth lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPERATING PROFIT after growth lead (owner draw already deducted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CASH AND SAFETY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment down payments (20% per new crew set)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash at year end (opening + profit - down payments)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before distributions beyond the owner draw and before income tax.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserve rule: 2 months of overhead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash must stay above this before any hire or purchase.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserve met?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WHAT THE COMPANY IS WORTH (indicative)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seller's discretionary earnings (operating profit + owner draw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SDE multiple (BizBuySell landscaping median 2021-25: 2.46x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recurring Drain Check revenue, documented systems and a manager who is not the owner all push toward the top of the range.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicative enterprise value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cross-check: revenue x 0.70 (BizBuySell). Not a promise; a benchmark.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sources and notes</t>
   </si>
   <si>
@@ -964,6 +1181,12 @@
   </si>
   <si>
     <t xml:space="preserve">Population ~35,700; median home value ~$411-423K; 56% owner-occupied; large 1970-1989 housing stock (original drainage aging out). https://www.city-data.com/zips/70808.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BizBuySell - Landscaping &amp; Yard Service valuation benchmarks (945 sold businesses, 2021-2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median sale price $425,000; median revenue $708,412; median SDE $187,761; revenue multiple 0.70x; SDE multiple 2.46x. https://www.bizbuysell.com/learning-center/valuation-benchmarks/landscaping-yard-service/</t>
   </si>
   <si>
     <t xml:space="preserve">BLS OEWS May 2023 - Baton Rouge MSA</t>
@@ -994,12 +1217,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="0.00"/>
+    <numFmt numFmtId="169" formatCode="@"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -1157,7 +1381,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1288,6 +1512,14 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -10334,7 +10566,1407 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:H53"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="29"/>
+      <c r="B4" s="29" t="s">
+        <v>298</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" s="29" t="s">
+        <v>146</v>
+      </c>
+      <c r="E4" s="29" t="s">
+        <v>299</v>
+      </c>
+      <c r="F4" s="29" t="s">
+        <v>300</v>
+      </c>
+      <c r="G4" s="29" t="s">
+        <v>301</v>
+      </c>
+      <c r="H4" s="29" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="s">
+        <v>304</v>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="s">
+        <v>306</v>
+      </c>
+      <c r="B7" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="21" t="n">
+        <f aca="false">(6*1+6*2)/12</f>
+        <v>1.5</v>
+      </c>
+      <c r="D7" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="33" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F7" s="33" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G7" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>4800</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <f aca="false">'Proforma 24 mo'!Z17/C7</f>
+        <v>9266.66666666667</v>
+      </c>
+      <c r="D8" s="25" t="n">
+        <f aca="false">'Proforma 24 mo'!AA17/D7</f>
+        <v>10800</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <f aca="false">Assumptions!$B$11*12*0.95</f>
+        <v>10260</v>
+      </c>
+      <c r="F8" s="25" t="n">
+        <f aca="false">Assumptions!$B$11*12*0.95</f>
+        <v>10260</v>
+      </c>
+      <c r="G8" s="25" t="n">
+        <f aca="false">Assumptions!$B$11*12*0.95</f>
+        <v>10260</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15" t="s">
+        <v>310</v>
+      </c>
+      <c r="B9" s="19" t="n">
+        <f aca="false">B7*B8</f>
+        <v>4800</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <f aca="false">'Proforma 24 mo'!Z17</f>
+        <v>13900</v>
+      </c>
+      <c r="D9" s="25" t="n">
+        <f aca="false">'Proforma 24 mo'!AA17</f>
+        <v>21600</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <f aca="false">E7*E8</f>
+        <v>25650</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <f aca="false">F7*F8</f>
+        <v>35910</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <f aca="false">G7*G8</f>
+        <v>41040</v>
+      </c>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="B11" s="26" t="n">
+        <f aca="false">Assumptions!$B$5</f>
+        <v>50</v>
+      </c>
+      <c r="C11" s="26" t="n">
+        <f aca="false">Assumptions!$B$5</f>
+        <v>50</v>
+      </c>
+      <c r="D11" s="26" t="n">
+        <f aca="false">Assumptions!$B$5</f>
+        <v>50</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <f aca="false">D11*1.03</f>
+        <v>51.5</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <f aca="false">E11*1.03</f>
+        <v>53.045</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <f aca="false">F11*1.03</f>
+        <v>54.63635</v>
+      </c>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="s">
+        <v>312</v>
+      </c>
+      <c r="B12" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!B25*12</f>
+        <v>380372.093023256</v>
+      </c>
+      <c r="C12" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z25</f>
+        <v>749744.186046512</v>
+      </c>
+      <c r="D12" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA25</f>
+        <v>1081674.41860465</v>
+      </c>
+      <c r="E12" s="22" t="n">
+        <f aca="false">E9*E11</f>
+        <v>1320975</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <f aca="false">F9*F11</f>
+        <v>1904845.95</v>
+      </c>
+      <c r="G12" s="22" t="n">
+        <f aca="false">G9*G11</f>
+        <v>2242275.804</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="25" t="n">
+        <f aca="false">'Proforma 24 mo'!M27</f>
+        <v>69.0010213081308</v>
+      </c>
+      <c r="D13" s="25" t="n">
+        <f aca="false">'Proforma 24 mo'!Y27</f>
+        <v>150.475943667911</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>260</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <v>380</v>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>480</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="s">
+        <v>316</v>
+      </c>
+      <c r="B14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z28</f>
+        <v>6875.46737058665</v>
+      </c>
+      <c r="D14" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA28</f>
+        <v>28691.7837941484</v>
+      </c>
+      <c r="E14" s="26" t="n">
+        <f aca="false">(D13+E13)/2*Assumptions!$B$28</f>
+        <v>51104.254986655</v>
+      </c>
+      <c r="F14" s="26" t="n">
+        <f aca="false">(E13+F13)/2*Assumptions!$B$28*1.03</f>
+        <v>82070.4</v>
+      </c>
+      <c r="G14" s="26" t="n">
+        <f aca="false">(F13+G13)/2*Assumptions!$B$28*1.06</f>
+        <v>113494.2</v>
+      </c>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="B15" s="23" t="n">
+        <f aca="false">B12+B14</f>
+        <v>380372.093023256</v>
+      </c>
+      <c r="C15" s="23" t="n">
+        <f aca="false">C12+C14</f>
+        <v>756619.653417098</v>
+      </c>
+      <c r="D15" s="23" t="n">
+        <f aca="false">D12+D14</f>
+        <v>1110366.2023988</v>
+      </c>
+      <c r="E15" s="23" t="n">
+        <f aca="false">E12+E14</f>
+        <v>1372079.25498666</v>
+      </c>
+      <c r="F15" s="23" t="n">
+        <f aca="false">F12+F14</f>
+        <v>1986916.35</v>
+      </c>
+      <c r="G15" s="23" t="n">
+        <f aca="false">G12+G14</f>
+        <v>2355770.004</v>
+      </c>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
+        <v>317</v>
+      </c>
+      <c r="B17" s="26" t="n">
+        <f aca="false">B7*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12</f>
+        <v>166848.12</v>
+      </c>
+      <c r="C17" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z32</f>
+        <v>250272.18</v>
+      </c>
+      <c r="D17" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA32</f>
+        <v>333696.24</v>
+      </c>
+      <c r="E17" s="26" t="n">
+        <f aca="false">E7*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03</f>
+        <v>429633.909</v>
+      </c>
+      <c r="F17" s="26" t="n">
+        <f aca="false">F7*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^2</f>
+        <v>619532.096778</v>
+      </c>
+      <c r="G17" s="26" t="n">
+        <f aca="false">G7*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^3</f>
+        <v>729277.78249296</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="B18" s="26" t="n">
+        <f aca="false">B12*Assumptions!$B$20</f>
+        <v>76074.4186046512</v>
+      </c>
+      <c r="C18" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z33</f>
+        <v>149948.837209302</v>
+      </c>
+      <c r="D18" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA33</f>
+        <v>216334.88372093</v>
+      </c>
+      <c r="E18" s="26" t="n">
+        <f aca="false">E12*Assumptions!$B$20</f>
+        <v>264195</v>
+      </c>
+      <c r="F18" s="26" t="n">
+        <f aca="false">F12*Assumptions!$B$20</f>
+        <v>380969.19</v>
+      </c>
+      <c r="G18" s="26" t="n">
+        <f aca="false">G12*Assumptions!$B$20</f>
+        <v>448455.1608</v>
+      </c>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="17" t="s">
+        <v>319</v>
+      </c>
+      <c r="B19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z34</f>
+        <v>1932.86231301633</v>
+      </c>
+      <c r="D19" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA34</f>
+        <v>8065.96331562404</v>
+      </c>
+      <c r="E19" s="26" t="n">
+        <f aca="false">E14/Assumptions!$B$28*Assumptions!$B$34</f>
+        <v>14366.6580283769</v>
+      </c>
+      <c r="F19" s="26" t="n">
+        <f aca="false">F14/Assumptions!$B$28/1.03*Assumptions!$B$34</f>
+        <v>22400</v>
+      </c>
+      <c r="G19" s="26" t="n">
+        <f aca="false">G14/Assumptions!$B$28/1.06*Assumptions!$B$34</f>
+        <v>30100</v>
+      </c>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="B20" s="23" t="n">
+        <f aca="false">B15-B17-B18-B19</f>
+        <v>137449.554418605</v>
+      </c>
+      <c r="C20" s="23" t="n">
+        <f aca="false">C15-C17-C18-C19</f>
+        <v>354465.77389478</v>
+      </c>
+      <c r="D20" s="23" t="n">
+        <f aca="false">D15-D17-D18-D19</f>
+        <v>552269.115362245</v>
+      </c>
+      <c r="E20" s="23" t="n">
+        <f aca="false">E15-E17-E18-E19</f>
+        <v>663883.687958278</v>
+      </c>
+      <c r="F20" s="23" t="n">
+        <f aca="false">F15-F17-F18-F19</f>
+        <v>964015.063222</v>
+      </c>
+      <c r="G20" s="23" t="n">
+        <f aca="false">G15-G17-G18-G19</f>
+        <v>1147937.06070704</v>
+      </c>
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="17" t="s">
+        <v>220</v>
+      </c>
+      <c r="B21" s="20" t="n">
+        <f aca="false">IF(B15=0,0,B20/B15)</f>
+        <v>0.361355517241379</v>
+      </c>
+      <c r="C21" s="20" t="n">
+        <f aca="false">IF(C15=0,0,C20/C15)</f>
+        <v>0.468486077904422</v>
+      </c>
+      <c r="D21" s="20" t="n">
+        <f aca="false">IF(D15=0,0,D20/D15)</f>
+        <v>0.497375653337737</v>
+      </c>
+      <c r="E21" s="20" t="n">
+        <f aca="false">IF(E15=0,0,E20/E15)</f>
+        <v>0.483852288813109</v>
+      </c>
+      <c r="F21" s="20" t="n">
+        <f aca="false">IF(F15=0,0,F20/F15)</f>
+        <v>0.485181504104086</v>
+      </c>
+      <c r="G21" s="20" t="n">
+        <f aca="false">IF(G15=0,0,G20/G15)</f>
+        <v>0.487287408685012</v>
+      </c>
+      <c r="H21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="B23" s="26" t="n">
+        <f aca="false">Assumptions!$B$55*12</f>
+        <v>72000</v>
+      </c>
+      <c r="C23" s="26" t="n">
+        <f aca="false">Assumptions!$B$55*12</f>
+        <v>72000</v>
+      </c>
+      <c r="D23" s="26" t="n">
+        <f aca="false">Assumptions!$B$55*12</f>
+        <v>72000</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>84000</v>
+      </c>
+      <c r="F23" s="9" t="n">
+        <v>96000</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>108000</v>
+      </c>
+      <c r="H23" s="7" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="17" t="s">
+        <v>322</v>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="9" t="n">
+        <v>24000</v>
+      </c>
+      <c r="E24" s="9" t="n">
+        <v>42000</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>48000</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="17" t="s">
+        <v>324</v>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>48750</v>
+      </c>
+      <c r="F25" s="9" t="n">
+        <v>70000</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>72000</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="17" t="s">
+        <v>326</v>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>55000</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>58000</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="17" t="s">
+        <v>328</v>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>18000</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="17" t="s">
+        <v>330</v>
+      </c>
+      <c r="B28" s="26" t="n">
+        <f aca="false">Assumptions!$B$56*12</f>
+        <v>10800</v>
+      </c>
+      <c r="C28" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z40</f>
+        <v>10800</v>
+      </c>
+      <c r="D28" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA40</f>
+        <v>10800</v>
+      </c>
+      <c r="E28" s="26" t="n">
+        <f aca="false">Assumptions!$B$56*12+9000*(E6-1)</f>
+        <v>28800</v>
+      </c>
+      <c r="F28" s="26" t="n">
+        <f aca="false">Assumptions!$B$56*12+9000*(F6-1)</f>
+        <v>37800</v>
+      </c>
+      <c r="G28" s="26" t="n">
+        <f aca="false">Assumptions!$B$56*12+9000*(G6-1)</f>
+        <v>37800</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="17" t="s">
+        <v>332</v>
+      </c>
+      <c r="B29" s="26" t="n">
+        <f aca="false">Assumptions!$B$57*12</f>
+        <v>21600</v>
+      </c>
+      <c r="C29" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z41+'Proforma 24 mo'!Z51</f>
+        <v>31015.9899306742</v>
+      </c>
+      <c r="D29" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA41+'Proforma 24 mo'!AA51</f>
+        <v>49200.3091089603</v>
+      </c>
+      <c r="E29" s="26" t="n">
+        <f aca="false">Assumptions!$B$57*12+'Equipment plan'!H10*12*(E6-1)</f>
+        <v>76800.6182179206</v>
+      </c>
+      <c r="F29" s="26" t="n">
+        <f aca="false">Assumptions!$B$57*12+'Equipment plan'!H10*12*(F6-1)</f>
+        <v>104400.927326881</v>
+      </c>
+      <c r="G29" s="26" t="n">
+        <f aca="false">Assumptions!$B$57*12+'Equipment plan'!H10*12*(G6-1)</f>
+        <v>104400.927326881</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="17" t="s">
+        <v>334</v>
+      </c>
+      <c r="B30" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="26" t="n">
+        <f aca="false">Assumptions!$B$61*12</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>25500</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>37800</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>50400</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>52000</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="17" t="s">
+        <v>336</v>
+      </c>
+      <c r="B31" s="26" t="n">
+        <f aca="false">Assumptions!$B$58*12</f>
+        <v>4200</v>
+      </c>
+      <c r="C31" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z42</f>
+        <v>4200</v>
+      </c>
+      <c r="D31" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA42</f>
+        <v>4200</v>
+      </c>
+      <c r="E31" s="22" t="n">
+        <f aca="false">4200+1200*E6</f>
+        <v>7800</v>
+      </c>
+      <c r="F31" s="22" t="n">
+        <f aca="false">4200+1200*F6</f>
+        <v>9000</v>
+      </c>
+      <c r="G31" s="22" t="n">
+        <f aca="false">4200+1200*G6</f>
+        <v>9000</v>
+      </c>
+      <c r="H31" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="17" t="s">
+        <v>337</v>
+      </c>
+      <c r="B32" s="26" t="n">
+        <f aca="false">Assumptions!$B$59*12</f>
+        <v>3000</v>
+      </c>
+      <c r="C32" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z43</f>
+        <v>3000</v>
+      </c>
+      <c r="D32" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA43</f>
+        <v>3000</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>7200</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>9600</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="17" t="s">
+        <v>339</v>
+      </c>
+      <c r="B33" s="26" t="n">
+        <f aca="false">(Assumptions!$B$41+Assumptions!$B$44+Assumptions!$B$53)*12</f>
+        <v>21600</v>
+      </c>
+      <c r="C33" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z47+'Proforma 24 mo'!Z48+'Proforma 24 mo'!Z49</f>
+        <v>26400</v>
+      </c>
+      <c r="D33" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA47+'Proforma 24 mo'!AA48+'Proforma 24 mo'!AA49</f>
+        <v>32400</v>
+      </c>
+      <c r="E33" s="22" t="n">
+        <f aca="false">E15*0.05</f>
+        <v>68603.9627493328</v>
+      </c>
+      <c r="F33" s="22" t="n">
+        <f aca="false">F15*0.05</f>
+        <v>99345.8175</v>
+      </c>
+      <c r="G33" s="22" t="n">
+        <f aca="false">G15*0.045</f>
+        <v>106009.65018</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="17" t="s">
+        <v>341</v>
+      </c>
+      <c r="B34" s="26" t="n">
+        <f aca="false">Assumptions!$B$60*12</f>
+        <v>7200</v>
+      </c>
+      <c r="C34" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z44</f>
+        <v>7200</v>
+      </c>
+      <c r="D34" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA44</f>
+        <v>7200</v>
+      </c>
+      <c r="E34" s="22" t="n">
+        <f aca="false">7200+3000*E6</f>
+        <v>16200</v>
+      </c>
+      <c r="F34" s="22" t="n">
+        <f aca="false">7200+3000*F6</f>
+        <v>19200</v>
+      </c>
+      <c r="G34" s="22" t="n">
+        <f aca="false">7200+3000*G6</f>
+        <v>19200</v>
+      </c>
+      <c r="H34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="17" t="s">
+        <v>342</v>
+      </c>
+      <c r="B35" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z50</f>
+        <v>15600</v>
+      </c>
+      <c r="D35" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA50</f>
+        <v>0</v>
+      </c>
+      <c r="E35" s="26" t="n">
+        <f aca="false">(E6-D6)*('Equipment plan'!E10+Assumptions!$B$82)</f>
+        <v>15600</v>
+      </c>
+      <c r="F35" s="26" t="n">
+        <f aca="false">(F6-E6)*('Equipment plan'!E10+Assumptions!$B$82)</f>
+        <v>15600</v>
+      </c>
+      <c r="G35" s="26" t="n">
+        <f aca="false">(G6-F6)*('Equipment plan'!E10+Assumptions!$B$82)</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="17" t="s">
+        <v>344</v>
+      </c>
+      <c r="B37" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="9" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D37" s="9" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>66000</v>
+      </c>
+      <c r="F37" s="9" t="n">
+        <v>72000</v>
+      </c>
+      <c r="G37" s="9" t="n">
+        <v>72000</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="17" t="s">
+        <v>346</v>
+      </c>
+      <c r="B38" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D38" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E38" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F38" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G38" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="17" t="s">
+        <v>348</v>
+      </c>
+      <c r="B39" s="22" t="n">
+        <f aca="false">MAX(0,B43)</f>
+        <v>0</v>
+      </c>
+      <c r="C39" s="22" t="n">
+        <f aca="false">MAX(0,B43)</f>
+        <v>0</v>
+      </c>
+      <c r="D39" s="22" t="n">
+        <f aca="false">MAX(0,B43)</f>
+        <v>0</v>
+      </c>
+      <c r="E39" s="22" t="n">
+        <f aca="false">MAX(0,B43)</f>
+        <v>0</v>
+      </c>
+      <c r="F39" s="22" t="n">
+        <f aca="false">MAX(0,B43)</f>
+        <v>0</v>
+      </c>
+      <c r="G39" s="22" t="n">
+        <f aca="false">MAX(0,B43)</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="17" t="s">
+        <v>350</v>
+      </c>
+      <c r="B40" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="22" t="n">
+        <f aca="false">C37+C38*MAX(0,C42-C39)</f>
+        <v>78424.9783964105</v>
+      </c>
+      <c r="D40" s="22" t="n">
+        <f aca="false">D37+D38*MAX(0,D42-D39)</f>
+        <v>91796.8806253285</v>
+      </c>
+      <c r="E40" s="22" t="n">
+        <f aca="false">E37+E38*MAX(0,E42-E39)</f>
+        <v>87832.9106991025</v>
+      </c>
+      <c r="F40" s="22" t="n">
+        <f aca="false">F37+F38*MAX(0,F42-F39)</f>
+        <v>105226.831839512</v>
+      </c>
+      <c r="G40" s="22" t="n">
+        <f aca="false">G37+G38*MAX(0,G42-G39)</f>
+        <v>122192.648320016</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="15" t="s">
+        <v>352</v>
+      </c>
+      <c r="B41" s="23" t="n">
+        <f aca="false">SUM(B23:B35)</f>
+        <v>140400</v>
+      </c>
+      <c r="C41" s="23" t="n">
+        <f aca="false">SUM(C23:C35)</f>
+        <v>170215.989930674</v>
+      </c>
+      <c r="D41" s="23" t="n">
+        <f aca="false">SUM(D23:D35)</f>
+        <v>234300.30910896</v>
+      </c>
+      <c r="E41" s="23" t="n">
+        <f aca="false">SUM(E23:E35)</f>
+        <v>445554.580967253</v>
+      </c>
+      <c r="F41" s="23" t="n">
+        <f aca="false">SUM(F23:F35)</f>
+        <v>631746.744826881</v>
+      </c>
+      <c r="G41" s="23" t="n">
+        <f aca="false">SUM(G23:G35)</f>
+        <v>646010.577506881</v>
+      </c>
+      <c r="H41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="15" t="s">
+        <v>353</v>
+      </c>
+      <c r="B42" s="23" t="n">
+        <f aca="false">B20-B41</f>
+        <v>-2950.44558139535</v>
+      </c>
+      <c r="C42" s="23" t="n">
+        <f aca="false">C20-C41</f>
+        <v>184249.783964105</v>
+      </c>
+      <c r="D42" s="23" t="n">
+        <f aca="false">D20-D41</f>
+        <v>317968.806253285</v>
+      </c>
+      <c r="E42" s="23" t="n">
+        <f aca="false">E20-E41</f>
+        <v>218329.106991025</v>
+      </c>
+      <c r="F42" s="23" t="n">
+        <f aca="false">F20-F41</f>
+        <v>332268.318395119</v>
+      </c>
+      <c r="G42" s="23" t="n">
+        <f aca="false">G20-G41</f>
+        <v>501926.483200159</v>
+      </c>
+      <c r="H42" s="2"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="15" t="s">
+        <v>354</v>
+      </c>
+      <c r="B43" s="23" t="n">
+        <f aca="false">B42-B40</f>
+        <v>-2950.44558139535</v>
+      </c>
+      <c r="C43" s="23" t="n">
+        <f aca="false">C42-C40</f>
+        <v>105824.805567695</v>
+      </c>
+      <c r="D43" s="23" t="n">
+        <f aca="false">D42-D40</f>
+        <v>226171.925627957</v>
+      </c>
+      <c r="E43" s="23" t="n">
+        <f aca="false">E42-E40</f>
+        <v>130496.196291922</v>
+      </c>
+      <c r="F43" s="23" t="n">
+        <f aca="false">F42-F40</f>
+        <v>227041.486555607</v>
+      </c>
+      <c r="G43" s="23" t="n">
+        <f aca="false">G42-G40</f>
+        <v>379733.834880143</v>
+      </c>
+      <c r="H43" s="2"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="B44" s="20" t="n">
+        <f aca="false">IF(B15=0,0,B43/B15)</f>
+        <v>-0.00775673514306678</v>
+      </c>
+      <c r="C44" s="20" t="n">
+        <f aca="false">IF(C15=0,0,C43/C15)</f>
+        <v>0.139865261349955</v>
+      </c>
+      <c r="D44" s="20" t="n">
+        <f aca="false">IF(D15=0,0,D43/D15)</f>
+        <v>0.203691291340949</v>
+      </c>
+      <c r="E44" s="20" t="n">
+        <f aca="false">IF(E15=0,0,E43/E15)</f>
+        <v>0.0951083516623765</v>
+      </c>
+      <c r="F44" s="20" t="n">
+        <f aca="false">IF(F15=0,0,F43/F15)</f>
+        <v>0.114268266278853</v>
+      </c>
+      <c r="G44" s="20" t="n">
+        <f aca="false">IF(G15=0,0,G43/G15)</f>
+        <v>0.161193085163395</v>
+      </c>
+      <c r="H44" s="2"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="17" t="s">
+        <v>356</v>
+      </c>
+      <c r="B46" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!Z58</f>
+        <v>27700</v>
+      </c>
+      <c r="D46" s="26" t="n">
+        <f aca="false">'Proforma 24 mo'!AA58</f>
+        <v>0</v>
+      </c>
+      <c r="E46" s="22" t="n">
+        <f aca="false">(E6-D6)*'Equipment plan'!G10</f>
+        <v>27700</v>
+      </c>
+      <c r="F46" s="22" t="n">
+        <f aca="false">(F6-E6)*'Equipment plan'!G10</f>
+        <v>27700</v>
+      </c>
+      <c r="G46" s="22" t="n">
+        <f aca="false">(G6-F6)*'Equipment plan'!G10</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="2"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="15" t="s">
+        <v>357</v>
+      </c>
+      <c r="B47" s="26" t="n">
+        <f aca="false">Assumptions!$B$39</f>
+        <v>25000</v>
+      </c>
+      <c r="C47" s="23" t="n">
+        <f aca="false">B47+C43-C46</f>
+        <v>103124.805567695</v>
+      </c>
+      <c r="D47" s="23" t="n">
+        <f aca="false">C47+D43-D46</f>
+        <v>329296.731195651</v>
+      </c>
+      <c r="E47" s="23" t="n">
+        <f aca="false">D47+E43-E46</f>
+        <v>432092.927487574</v>
+      </c>
+      <c r="F47" s="23" t="n">
+        <f aca="false">E47+F43-F46</f>
+        <v>631434.414043181</v>
+      </c>
+      <c r="G47" s="23" t="n">
+        <f aca="false">F47+G43-G46</f>
+        <v>1011168.24892332</v>
+      </c>
+      <c r="H47" s="7" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="17" t="s">
+        <v>359</v>
+      </c>
+      <c r="B48" s="22" t="n">
+        <f aca="false">B41/6</f>
+        <v>23400</v>
+      </c>
+      <c r="C48" s="22" t="n">
+        <f aca="false">C41/6</f>
+        <v>28369.3316551124</v>
+      </c>
+      <c r="D48" s="22" t="n">
+        <f aca="false">D41/6</f>
+        <v>39050.0515181601</v>
+      </c>
+      <c r="E48" s="22" t="n">
+        <f aca="false">E41/6</f>
+        <v>74259.0968278756</v>
+      </c>
+      <c r="F48" s="22" t="n">
+        <f aca="false">F41/6</f>
+        <v>105291.124137813</v>
+      </c>
+      <c r="G48" s="22" t="n">
+        <f aca="false">G41/6</f>
+        <v>107668.42958448</v>
+      </c>
+      <c r="H48" s="7" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="B49" s="34" t="str">
+        <f aca="false">IF(B47&gt;=B48,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="C49" s="34" t="str">
+        <f aca="false">IF(C47&gt;=C48,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="D49" s="34" t="str">
+        <f aca="false">IF(D47&gt;=D48,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="E49" s="34" t="str">
+        <f aca="false">IF(E47&gt;=E48,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="F49" s="34" t="str">
+        <f aca="false">IF(F47&gt;=F48,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="G49" s="34" t="str">
+        <f aca="false">IF(G47&gt;=G48,"yes","NO")</f>
+        <v>yes</v>
+      </c>
+      <c r="H49" s="2"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="B50" s="5"/>
+      <c r="C50" s="5"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="17" t="s">
+        <v>363</v>
+      </c>
+      <c r="B51" s="22" t="n">
+        <f aca="false">B43+B23</f>
+        <v>69049.5544186047</v>
+      </c>
+      <c r="C51" s="22" t="n">
+        <f aca="false">C43+C23</f>
+        <v>177824.805567695</v>
+      </c>
+      <c r="D51" s="22" t="n">
+        <f aca="false">D43+D23</f>
+        <v>298171.925627957</v>
+      </c>
+      <c r="E51" s="22" t="n">
+        <f aca="false">E43+E23</f>
+        <v>214496.196291922</v>
+      </c>
+      <c r="F51" s="22" t="n">
+        <f aca="false">F43+F23</f>
+        <v>323041.486555607</v>
+      </c>
+      <c r="G51" s="22" t="n">
+        <f aca="false">G43+G23</f>
+        <v>487733.834880143</v>
+      </c>
+      <c r="H51" s="2"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="17" t="s">
+        <v>364</v>
+      </c>
+      <c r="B52" s="33" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="C52" s="33" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="D52" s="33" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="E52" s="33" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="F52" s="33" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="G52" s="33" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="H52" s="7" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="15" t="s">
+        <v>366</v>
+      </c>
+      <c r="B53" s="23" t="n">
+        <f aca="false">B51*B52</f>
+        <v>169861.903869767</v>
+      </c>
+      <c r="C53" s="23" t="n">
+        <f aca="false">C51*C52</f>
+        <v>437449.021696529</v>
+      </c>
+      <c r="D53" s="23" t="n">
+        <f aca="false">D51*D52</f>
+        <v>733502.937044773</v>
+      </c>
+      <c r="E53" s="23" t="n">
+        <f aca="false">E51*E52</f>
+        <v>527660.642878129</v>
+      </c>
+      <c r="F53" s="23" t="n">
+        <f aca="false">F51*F52</f>
+        <v>794682.056926794</v>
+      </c>
+      <c r="G53" s="23" t="n">
+        <f aca="false">G51*G52</f>
+        <v>1199825.23380515</v>
+      </c>
+      <c r="H53" s="7" t="s">
+        <v>367</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
@@ -10343,7 +11975,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>296</v>
+        <v>368</v>
       </c>
       <c r="B1" s="2"/>
     </row>
@@ -10352,99 +11984,107 @@
       <c r="B2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="33" t="s">
-        <v>297</v>
-      </c>
-      <c r="B3" s="34" t="s">
-        <v>298</v>
+      <c r="A3" s="35" t="s">
+        <v>369</v>
+      </c>
+      <c r="B3" s="36" t="s">
+        <v>370</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="33" t="s">
-        <v>299</v>
-      </c>
-      <c r="B4" s="34" t="s">
-        <v>300</v>
+      <c r="A4" s="35" t="s">
+        <v>371</v>
+      </c>
+      <c r="B4" s="36" t="s">
+        <v>372</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="33" t="s">
-        <v>301</v>
-      </c>
-      <c r="B5" s="34" t="s">
-        <v>302</v>
+      <c r="A5" s="35" t="s">
+        <v>373</v>
+      </c>
+      <c r="B5" s="36" t="s">
+        <v>374</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="33" t="s">
-        <v>303</v>
-      </c>
-      <c r="B6" s="34" t="s">
-        <v>304</v>
+      <c r="A6" s="35" t="s">
+        <v>375</v>
+      </c>
+      <c r="B6" s="36" t="s">
+        <v>376</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="33" t="s">
-        <v>305</v>
-      </c>
-      <c r="B7" s="34" t="s">
-        <v>306</v>
+      <c r="A7" s="35" t="s">
+        <v>377</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>378</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="33" t="s">
-        <v>307</v>
-      </c>
-      <c r="B8" s="34" t="s">
-        <v>308</v>
+      <c r="A8" s="35" t="s">
+        <v>379</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>380</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="33" t="s">
-        <v>309</v>
-      </c>
-      <c r="B9" s="34" t="s">
-        <v>310</v>
+      <c r="A9" s="35" t="s">
+        <v>381</v>
+      </c>
+      <c r="B9" s="36" t="s">
+        <v>382</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="33" t="s">
-        <v>311</v>
-      </c>
-      <c r="B10" s="34" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="33" t="s">
-        <v>313</v>
-      </c>
-      <c r="B11" s="34" t="s">
-        <v>314</v>
+      <c r="A10" s="35" t="s">
+        <v>383</v>
+      </c>
+      <c r="B10" s="36" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="35" t="s">
+        <v>385</v>
+      </c>
+      <c r="B11" s="36" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="33" t="s">
-        <v>315</v>
-      </c>
-      <c r="B12" s="34" t="s">
-        <v>316</v>
+      <c r="A12" s="35" t="s">
+        <v>387</v>
+      </c>
+      <c r="B12" s="36" t="s">
+        <v>388</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="33" t="s">
-        <v>317</v>
-      </c>
-      <c r="B13" s="34" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="33" t="s">
-        <v>319</v>
-      </c>
-      <c r="B14" s="34" t="s">
-        <v>320</v>
+      <c r="A13" s="35" t="s">
+        <v>389</v>
+      </c>
+      <c r="B13" s="36" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="35" t="s">
+        <v>391</v>
+      </c>
+      <c r="B14" s="36" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="35" t="s">
+        <v>393</v>
+      </c>
+      <c r="B15" s="36" t="s">
+        <v>394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: three-case model (worst/conservative/strong), 90-day execution plan, operating rhythm, ownership and exit terms
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LoK8Mi2K1W9PhhoHM3MdEb
</commit_message>
<xml_diff>
--- a/docs/Scag-Scapes-Proforma.xlsx
+++ b/docs/Scag-Scapes-Proforma.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Scenarios" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Equipment plan" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="5-year plan" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Sources &amp; notes" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Three cases 5-yr" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Sources &amp; notes" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="463">
   <si>
     <t xml:space="preserve">Scag Scapes LLC - Growth Proforma - Assumptions</t>
   </si>
@@ -1157,6 +1158,183 @@
   </si>
   <si>
     <t xml:space="preserve">Cross-check: revenue x 0.70 (BizBuySell). Not a promise; a benchmark.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worst case, conservative, strong - the same business run three ways</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue = change it. The middle block is the plan in the blueprint. Today's run rate is on the '5-year plan' tab and is the same in all three cases; what differs is only how fast crews fill their days, what a foot sells for, how many plans attach, and when a crew is added.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Side by side</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worst case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue - year 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue - year 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linear feet installed - year 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gross margin - year 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operating profit before the growth lead - year 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operating profit after the growth lead - year 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operating profit after the growth lead - year 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What the growth lead costs - year 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What the growth lead costs - year 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner's cash from the business - year 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash at the end of year 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicative value at the end of year 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read it this way: plan around the worst case. There the 90-day gate ends the growth-lead arrangement for $15,000 and the company ends up roughly where it is today - that is the floor. The middle block is what the blueprint commits to. The right-hand block is the same plan with the levers landing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WORST CASE - most of it does not work</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leads cost more and close worse, crews never beat 36 LF a day, Crew 2 slips to the middle of year 2, few plans attach. The 90-day gate is missed, so the growth lead is ended after three months (that is the $15,000 in year 1 - the whole exposure) and no share is ever earned. The company then looks much like it does today: it covers itself and pays the owner, and it does not run away from anyone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drivers - change any blue cell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Half a crew = started mid-year. A crew is added only after three months at target, backlog over four weeks and cash above two months of overhead.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of crew days on drainage (the rest is pads, fences, sod, patios)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Today one crew spends about 42% of its days on drain feet. Filling the calendar is the whole growth engine.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LF a crew installs per working day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charlie's target is 43 (900 LF / 21 days).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual price change from year 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drain Check plans active at year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marketing as a share of revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overhead per crew per year (insurance, tools, uniforms, phones)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Office admin, operations manager, estimator, bonus pool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hired in that order, each before the crew that needs it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew days worked</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linear feet installed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drainage revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other work on the remaining days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew labor (wages from the Assumptions tab, +3% a year from year 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materials, fuel and plan visit costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overhead (owner draw, fixed costs, per crew, staff, marketing, yard, equipment loans)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner draw, existing payments, software, CPA, shop and the yard (sq ft x rate) all come from the Assumptions tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operating profit before the growth lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth lead - base for the year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set any year to 0 to see the plan without it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth lead - share of profit above today's baseline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Earned only on profit above what the business makes today.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth lead - total cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPERATING PROFIT after the growth lead</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operating margin (the owner draw is already paid)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment down payments for new crews</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash at year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before income tax and before any distribution beyond the owner draw. A falling line means the owner draw is larger than the business earns - the draw is a blue cell.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Owner's cash from the business (operating profit + owner draw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicative value at 2.46x SDE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BizBuySell landscaping median, 945 sales 2021-2025. A benchmark, not a promise.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONSERVATIVE - the plan in the blueprint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charlie's own targets on the blueprint's schedule: 900 LF a crew a month, 70% close, 40% plan attach, Crew 3 in year 3 and Crew 4 in year 4 - each only after its gate. This is an annual approximation of the 24-month proforma and lands within about 4% of it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STRONG - the levers work</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviews, referrals and the Moasure map support a 3% price step each year, crews settle at 48 LF a day, the plan book compounds and HOA / property-manager work fills the winter. Note the gross margin runs above Charlie's 50% rule - that is what productivity does to a fixed crew cost.</t>
   </si>
   <si>
     <t xml:space="preserve">Sources and notes</t>
@@ -1253,7 +1431,7 @@
     <numFmt numFmtId="169" formatCode="\$0.00"/>
     <numFmt numFmtId="170" formatCode="@"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1339,6 +1517,14 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF46524E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1409,7 +1595,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1565,6 +1751,22 @@
     <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
@@ -12114,6 +12316,2883 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:H122"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="56"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="5"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="16"/>
+      <c r="B5" s="29" t="s">
+        <v>380</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>257</v>
+      </c>
+      <c r="D5" s="29" t="s">
+        <v>381</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="B6" s="15" t="n">
+        <f aca="false">B39</f>
+        <v>359125.8</v>
+      </c>
+      <c r="C6" s="15" t="n">
+        <f aca="false">B73</f>
+        <v>721206</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <f aca="false">B107</f>
+        <v>881074.8</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
+        <v>383</v>
+      </c>
+      <c r="B7" s="15" t="n">
+        <f aca="false">F39</f>
+        <v>644276.4</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <f aca="false">F73</f>
+        <v>2487162.5583804</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <f aca="false">F107</f>
+        <v>3237506.55996845</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="B8" s="19" t="n">
+        <f aca="false">F35</f>
+        <v>11566.8</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <f aca="false">F69</f>
+        <v>41176.8</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <f aca="false">F103</f>
+        <v>51710.4</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="B9" s="21" t="n">
+        <f aca="false">F43</f>
+        <v>0.358714949844654</v>
+      </c>
+      <c r="C9" s="21" t="n">
+        <f aca="false">F77</f>
+        <v>0.494088304198659</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <f aca="false">F111</f>
+        <v>0.535112619981201</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>386</v>
+      </c>
+      <c r="B10" s="15" t="n">
+        <f aca="false">B45</f>
+        <v>-64486.915</v>
+      </c>
+      <c r="C10" s="15" t="n">
+        <f aca="false">B79</f>
+        <v>108938.36544552</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <f aca="false">B113</f>
+        <v>220821.13944552</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="16" t="s">
+        <v>387</v>
+      </c>
+      <c r="B11" s="23" t="n">
+        <f aca="false">B49</f>
+        <v>-79486.915</v>
+      </c>
+      <c r="C11" s="23" t="n">
+        <f aca="false">B83</f>
+        <v>38044.5289009678</v>
+      </c>
+      <c r="D11" s="23" t="n">
+        <f aca="false">B117</f>
+        <v>138739.025500968</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="s">
+        <v>388</v>
+      </c>
+      <c r="B12" s="23" t="n">
+        <f aca="false">F49</f>
+        <v>-44509.308042386</v>
+      </c>
+      <c r="C12" s="23" t="n">
+        <f aca="false">F83</f>
+        <v>468196.987941603</v>
+      </c>
+      <c r="D12" s="23" t="n">
+        <f aca="false">F117</f>
+        <v>798877.56638799</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="B13" s="15" t="n">
+        <f aca="false">B48</f>
+        <v>15000</v>
+      </c>
+      <c r="C13" s="15" t="n">
+        <f aca="false">B82</f>
+        <v>70893.836544552</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <f aca="false">B116</f>
+        <v>82082.113944552</v>
+      </c>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
+        <v>390</v>
+      </c>
+      <c r="B14" s="15" t="n">
+        <f aca="false">F48</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="15" t="n">
+        <f aca="false">F82</f>
+        <v>132021.887549067</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <f aca="false">F116</f>
+        <v>168764.17404311</v>
+      </c>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
+        <v>391</v>
+      </c>
+      <c r="B15" s="23" t="n">
+        <f aca="false">F53</f>
+        <v>27490.691957614</v>
+      </c>
+      <c r="C15" s="23" t="n">
+        <f aca="false">F87</f>
+        <v>540196.987941603</v>
+      </c>
+      <c r="D15" s="23" t="n">
+        <f aca="false">F121</f>
+        <v>870877.56638799</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="B16" s="15" t="n">
+        <f aca="false">F52</f>
+        <v>-220618.989948206</v>
+      </c>
+      <c r="C16" s="15" t="n">
+        <f aca="false">F86</f>
+        <v>1165532.33955517</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <f aca="false">F120</f>
+        <v>2443286.01286937</v>
+      </c>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
+        <v>393</v>
+      </c>
+      <c r="B17" s="23" t="n">
+        <f aca="false">F54</f>
+        <v>67627.1022157304</v>
+      </c>
+      <c r="C17" s="23" t="n">
+        <f aca="false">F88</f>
+        <v>1328884.59033634</v>
+      </c>
+      <c r="D17" s="23" t="n">
+        <f aca="false">F122</f>
+        <v>2142358.81331445</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="39" t="s">
+        <v>394</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="40" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="B23" s="29" t="s">
+        <v>151</v>
+      </c>
+      <c r="C23" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="D23" s="29" t="s">
+        <v>305</v>
+      </c>
+      <c r="E23" s="29" t="s">
+        <v>306</v>
+      </c>
+      <c r="F23" s="29" t="s">
+        <v>307</v>
+      </c>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="B24" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E24" s="33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F24" s="33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G24" s="2"/>
+      <c r="H24" s="7" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18" t="s">
+        <v>399</v>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C25" s="13" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D25" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E25" s="13" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G25" s="2"/>
+      <c r="H25" s="7" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18" t="s">
+        <v>401</v>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="D26" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="E26" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="F26" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="7" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="C27" s="15" t="n">
+        <f aca="false">B27*(1+$B$28)</f>
+        <v>48</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <f aca="false">C27*(1+$B$28)</f>
+        <v>48</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <f aca="false">D27*(1+$B$28)</f>
+        <v>48</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <f aca="false">E27*(1+$B$28)</f>
+        <v>48</v>
+      </c>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="18" t="s">
+        <v>403</v>
+      </c>
+      <c r="B28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="18" t="s">
+        <v>404</v>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>85</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>110</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>130</v>
+      </c>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="s">
+        <v>405</v>
+      </c>
+      <c r="B30" s="13" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="C30" s="13" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="D30" s="13" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="s">
+        <v>406</v>
+      </c>
+      <c r="B31" s="9" t="n">
+        <v>24000</v>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>24000</v>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>24000</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F31" s="9" t="n">
+        <v>24000</v>
+      </c>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="B32" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>24000</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>42000</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>44000</v>
+      </c>
+      <c r="G32" s="2"/>
+      <c r="H32" s="7" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="41" t="s">
+        <v>409</v>
+      </c>
+      <c r="B33" s="42"/>
+      <c r="C33" s="42"/>
+      <c r="D33" s="42"/>
+      <c r="E33" s="42"/>
+      <c r="F33" s="42"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="42"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="18" t="s">
+        <v>410</v>
+      </c>
+      <c r="B34" s="19" t="n">
+        <f aca="false">B24*Assumptions!$B$8*12</f>
+        <v>252</v>
+      </c>
+      <c r="C34" s="19" t="n">
+        <f aca="false">C24*Assumptions!$B$8*12</f>
+        <v>252</v>
+      </c>
+      <c r="D34" s="19" t="n">
+        <f aca="false">D24*Assumptions!$B$8*12</f>
+        <v>378</v>
+      </c>
+      <c r="E34" s="19" t="n">
+        <f aca="false">E24*Assumptions!$B$8*12</f>
+        <v>378</v>
+      </c>
+      <c r="F34" s="19" t="n">
+        <f aca="false">F24*Assumptions!$B$8*12</f>
+        <v>378</v>
+      </c>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="16" t="s">
+        <v>411</v>
+      </c>
+      <c r="B35" s="20" t="n">
+        <f aca="false">B34*B25*B26</f>
+        <v>4989.6</v>
+      </c>
+      <c r="C35" s="20" t="n">
+        <f aca="false">C34*C25*C26</f>
+        <v>6350.4</v>
+      </c>
+      <c r="D35" s="20" t="n">
+        <f aca="false">D34*D25*D26</f>
+        <v>10886.4</v>
+      </c>
+      <c r="E35" s="20" t="n">
+        <f aca="false">E34*E25*E26</f>
+        <v>11566.8</v>
+      </c>
+      <c r="F35" s="20" t="n">
+        <f aca="false">F34*F25*F26</f>
+        <v>11566.8</v>
+      </c>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="B36" s="15" t="n">
+        <f aca="false">B35*B27</f>
+        <v>239500.8</v>
+      </c>
+      <c r="C36" s="15" t="n">
+        <f aca="false">C35*C27</f>
+        <v>304819.2</v>
+      </c>
+      <c r="D36" s="15" t="n">
+        <f aca="false">D35*D27</f>
+        <v>522547.2</v>
+      </c>
+      <c r="E36" s="15" t="n">
+        <f aca="false">E35*E27</f>
+        <v>555206.4</v>
+      </c>
+      <c r="F36" s="15" t="n">
+        <f aca="false">F35*F27</f>
+        <v>555206.4</v>
+      </c>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="B37" s="15" t="n">
+        <f aca="false">B34*(1-B25)*Assumptions!$B$10</f>
+        <v>113400</v>
+      </c>
+      <c r="C37" s="15" t="n">
+        <f aca="false">C34*(1-C25)*Assumptions!$B$10</f>
+        <v>75600</v>
+      </c>
+      <c r="D37" s="15" t="n">
+        <f aca="false">D34*(1-D25)*Assumptions!$B$10</f>
+        <v>75600</v>
+      </c>
+      <c r="E37" s="15" t="n">
+        <f aca="false">E34*(1-E25)*Assumptions!$B$10</f>
+        <v>56700</v>
+      </c>
+      <c r="F37" s="15" t="n">
+        <f aca="false">F34*(1-F25)*Assumptions!$B$10</f>
+        <v>56700</v>
+      </c>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="B38" s="15" t="n">
+        <f aca="false">B29*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>6225</v>
+      </c>
+      <c r="C38" s="15" t="n">
+        <f aca="false">C29*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>13695</v>
+      </c>
+      <c r="D38" s="15" t="n">
+        <f aca="false">D29*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>21165</v>
+      </c>
+      <c r="E38" s="15" t="n">
+        <f aca="false">E29*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>27390</v>
+      </c>
+      <c r="F38" s="15" t="n">
+        <f aca="false">F29*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>32370</v>
+      </c>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="B39" s="23" t="n">
+        <f aca="false">B36+B37+B38</f>
+        <v>359125.8</v>
+      </c>
+      <c r="C39" s="23" t="n">
+        <f aca="false">C36+C37+C38</f>
+        <v>394114.2</v>
+      </c>
+      <c r="D39" s="23" t="n">
+        <f aca="false">D36+D37+D38</f>
+        <v>619312.2</v>
+      </c>
+      <c r="E39" s="23" t="n">
+        <f aca="false">E36+E37+E38</f>
+        <v>639296.4</v>
+      </c>
+      <c r="F39" s="23" t="n">
+        <f aca="false">F36+F37+F38</f>
+        <v>644276.4</v>
+      </c>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="18" t="s">
+        <v>414</v>
+      </c>
+      <c r="B40" s="15" t="n">
+        <f aca="false">B24*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(B1)-2)</f>
+        <v>166848.12</v>
+      </c>
+      <c r="C40" s="15" t="n">
+        <f aca="false">C24*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(C1)-2)</f>
+        <v>171853.5636</v>
+      </c>
+      <c r="D40" s="15" t="n">
+        <f aca="false">D24*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(D1)-2)</f>
+        <v>265513.755762</v>
+      </c>
+      <c r="E40" s="15" t="n">
+        <f aca="false">E24*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(E1)-2)</f>
+        <v>273479.16843486</v>
+      </c>
+      <c r="F40" s="15" t="n">
+        <f aca="false">F24*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(F1)-2)</f>
+        <v>281683.543487906</v>
+      </c>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="18" t="s">
+        <v>415</v>
+      </c>
+      <c r="B41" s="15" t="n">
+        <f aca="false">(B36+B37)*Assumptions!$B$20+B29/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>72330.16</v>
+      </c>
+      <c r="C41" s="15" t="n">
+        <f aca="false">(C36+C37)*Assumptions!$B$20+C29/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>79933.84</v>
+      </c>
+      <c r="D41" s="15" t="n">
+        <f aca="false">(D36+D37)*Assumptions!$B$20+D29/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>125579.44</v>
+      </c>
+      <c r="E41" s="15" t="n">
+        <f aca="false">(E36+E37)*Assumptions!$B$20+E29/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>130081.28</v>
+      </c>
+      <c r="F41" s="15" t="n">
+        <f aca="false">(F36+F37)*Assumptions!$B$20+F29/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>131481.28</v>
+      </c>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="B42" s="23" t="n">
+        <f aca="false">B39-B40-B41</f>
+        <v>119947.52</v>
+      </c>
+      <c r="C42" s="23" t="n">
+        <f aca="false">C39-C40-C41</f>
+        <v>142326.7964</v>
+      </c>
+      <c r="D42" s="23" t="n">
+        <f aca="false">D39-D40-D41</f>
+        <v>228219.004238</v>
+      </c>
+      <c r="E42" s="23" t="n">
+        <f aca="false">E39-E40-E41</f>
+        <v>235735.95156514</v>
+      </c>
+      <c r="F42" s="23" t="n">
+        <f aca="false">F39-F40-F41</f>
+        <v>231111.576512094</v>
+      </c>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="B43" s="21" t="n">
+        <f aca="false">IF(B39=0,0,B42/B39)</f>
+        <v>0.333998615526927</v>
+      </c>
+      <c r="C43" s="21" t="n">
+        <f aca="false">IF(C39=0,0,C42/C39)</f>
+        <v>0.361130850905651</v>
+      </c>
+      <c r="D43" s="21" t="n">
+        <f aca="false">IF(D39=0,0,D42/D39)</f>
+        <v>0.368503969787774</v>
+      </c>
+      <c r="E43" s="21" t="n">
+        <f aca="false">IF(E39=0,0,E42/E39)</f>
+        <v>0.368742810948317</v>
+      </c>
+      <c r="F43" s="21" t="n">
+        <f aca="false">IF(F39=0,0,F42/F39)</f>
+        <v>0.358714949844654</v>
+      </c>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="18" t="s">
+        <v>416</v>
+      </c>
+      <c r="B44" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+B24*B31+B32+B39*B30+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,B24-1)</f>
+        <v>184434.435</v>
+      </c>
+      <c r="C44" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+C24*C31+C32+C39*C30+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,C24-1)</f>
+        <v>187058.565</v>
+      </c>
+      <c r="D44" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+D24*D31+D32+D39*D30+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,D24-1)</f>
+        <v>253748.56955448</v>
+      </c>
+      <c r="E44" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+E24*E31+E32+E39*E30+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,E24-1)</f>
+        <v>273247.38455448</v>
+      </c>
+      <c r="F44" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+F24*F31+F32+F39*F30+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,F24-1)</f>
+        <v>275620.88455448</v>
+      </c>
+      <c r="G44" s="2"/>
+      <c r="H44" s="7" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="16" t="s">
+        <v>418</v>
+      </c>
+      <c r="B45" s="23" t="n">
+        <f aca="false">B42-B44</f>
+        <v>-64486.915</v>
+      </c>
+      <c r="C45" s="23" t="n">
+        <f aca="false">C42-C44</f>
+        <v>-44731.7686000001</v>
+      </c>
+      <c r="D45" s="23" t="n">
+        <f aca="false">D42-D44</f>
+        <v>-25529.5653164801</v>
+      </c>
+      <c r="E45" s="23" t="n">
+        <f aca="false">E42-E44</f>
+        <v>-37511.4329893402</v>
+      </c>
+      <c r="F45" s="23" t="n">
+        <f aca="false">F42-F44</f>
+        <v>-44509.308042386</v>
+      </c>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="B46" s="9" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C46" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="2"/>
+      <c r="H46" s="7" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="18" t="s">
+        <v>421</v>
+      </c>
+      <c r="B47" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C47" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D47" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E47" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F47" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G47" s="2"/>
+      <c r="H47" s="7" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="18" t="s">
+        <v>423</v>
+      </c>
+      <c r="B48" s="15" t="n">
+        <f aca="false">B46+IF(B46=0,0,B47*MAX(0,B45-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>15000</v>
+      </c>
+      <c r="C48" s="15" t="n">
+        <f aca="false">C46+IF(C46=0,0,C47*MAX(0,C45-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>0</v>
+      </c>
+      <c r="D48" s="15" t="n">
+        <f aca="false">D46+IF(D46=0,0,D47*MAX(0,D45-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>0</v>
+      </c>
+      <c r="E48" s="15" t="n">
+        <f aca="false">E46+IF(E46=0,0,E47*MAX(0,E45-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>0</v>
+      </c>
+      <c r="F48" s="15" t="n">
+        <f aca="false">F46+IF(F46=0,0,F47*MAX(0,F45-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>0</v>
+      </c>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="16" t="s">
+        <v>424</v>
+      </c>
+      <c r="B49" s="23" t="n">
+        <f aca="false">B45-B48</f>
+        <v>-79486.915</v>
+      </c>
+      <c r="C49" s="23" t="n">
+        <f aca="false">C45-C48</f>
+        <v>-44731.7686000001</v>
+      </c>
+      <c r="D49" s="23" t="n">
+        <f aca="false">D45-D48</f>
+        <v>-25529.5653164801</v>
+      </c>
+      <c r="E49" s="23" t="n">
+        <f aca="false">E45-E48</f>
+        <v>-37511.4329893402</v>
+      </c>
+      <c r="F49" s="23" t="n">
+        <f aca="false">F45-F48</f>
+        <v>-44509.308042386</v>
+      </c>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="18" t="s">
+        <v>425</v>
+      </c>
+      <c r="B50" s="21" t="n">
+        <f aca="false">IF(B39=0,0,B49/B39)</f>
+        <v>-0.221334459958043</v>
+      </c>
+      <c r="C50" s="21" t="n">
+        <f aca="false">IF(C39=0,0,C49/C39)</f>
+        <v>-0.113499510040491</v>
+      </c>
+      <c r="D50" s="21" t="n">
+        <f aca="false">IF(D39=0,0,D49/D39)</f>
+        <v>-0.0412224485751776</v>
+      </c>
+      <c r="E50" s="21" t="n">
+        <f aca="false">IF(E39=0,0,E49/E39)</f>
+        <v>-0.0586761211064855</v>
+      </c>
+      <c r="F50" s="21" t="n">
+        <f aca="false">IF(F39=0,0,F49/F39)</f>
+        <v>-0.0690841819479745</v>
+      </c>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="18" t="s">
+        <v>426</v>
+      </c>
+      <c r="B51" s="15" t="n">
+        <f aca="false">MAX(0,B24-1)*'Equipment plan'!$G$10</f>
+        <v>0</v>
+      </c>
+      <c r="C51" s="15" t="n">
+        <f aca="false">MAX(0,C24-B24)*'Equipment plan'!$G$10</f>
+        <v>0</v>
+      </c>
+      <c r="D51" s="15" t="n">
+        <f aca="false">MAX(0,D24-C24)*'Equipment plan'!$G$10</f>
+        <v>13850</v>
+      </c>
+      <c r="E51" s="15" t="n">
+        <f aca="false">MAX(0,E24-D24)*'Equipment plan'!$G$10</f>
+        <v>0</v>
+      </c>
+      <c r="F51" s="15" t="n">
+        <f aca="false">MAX(0,F24-E24)*'Equipment plan'!$G$10</f>
+        <v>0</v>
+      </c>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="16" t="s">
+        <v>427</v>
+      </c>
+      <c r="B52" s="23" t="n">
+        <f aca="false">Assumptions!$B$39+B49-B51</f>
+        <v>-54486.915</v>
+      </c>
+      <c r="C52" s="23" t="n">
+        <f aca="false">B52+C49-C51</f>
+        <v>-99218.6836000001</v>
+      </c>
+      <c r="D52" s="23" t="n">
+        <f aca="false">C52+D49-D51</f>
+        <v>-138598.24891648</v>
+      </c>
+      <c r="E52" s="23" t="n">
+        <f aca="false">D52+E49-E51</f>
+        <v>-176109.68190582</v>
+      </c>
+      <c r="F52" s="23" t="n">
+        <f aca="false">E52+F49-F51</f>
+        <v>-220618.989948206</v>
+      </c>
+      <c r="G52" s="2"/>
+      <c r="H52" s="7" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="B53" s="15" t="n">
+        <f aca="false">B49+Assumptions!$B$55*12</f>
+        <v>-7486.91500000004</v>
+      </c>
+      <c r="C53" s="15" t="n">
+        <f aca="false">C49+Assumptions!$B$55*12</f>
+        <v>27268.2313999999</v>
+      </c>
+      <c r="D53" s="15" t="n">
+        <f aca="false">D49+Assumptions!$B$55*12</f>
+        <v>46470.4346835199</v>
+      </c>
+      <c r="E53" s="15" t="n">
+        <f aca="false">E49+Assumptions!$B$55*12</f>
+        <v>34488.5670106598</v>
+      </c>
+      <c r="F53" s="15" t="n">
+        <f aca="false">F49+Assumptions!$B$55*12</f>
+        <v>27490.691957614</v>
+      </c>
+      <c r="G53" s="2"/>
+      <c r="H53" s="2"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="18" t="s">
+        <v>430</v>
+      </c>
+      <c r="B54" s="15" t="n">
+        <f aca="false">MAX(0,B53)*2.46</f>
+        <v>0</v>
+      </c>
+      <c r="C54" s="15" t="n">
+        <f aca="false">MAX(0,C53)*2.46</f>
+        <v>67079.8492439998</v>
+      </c>
+      <c r="D54" s="15" t="n">
+        <f aca="false">MAX(0,D53)*2.46</f>
+        <v>114317.269321459</v>
+      </c>
+      <c r="E54" s="15" t="n">
+        <f aca="false">MAX(0,E53)*2.46</f>
+        <v>84841.8748462231</v>
+      </c>
+      <c r="F54" s="15" t="n">
+        <f aca="false">MAX(0,F53)*2.46</f>
+        <v>67627.1022157304</v>
+      </c>
+      <c r="G54" s="2"/>
+      <c r="H54" s="7" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+    </row>
+    <row r="56" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="40" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="B57" s="29" t="s">
+        <v>151</v>
+      </c>
+      <c r="C57" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="D57" s="29" t="s">
+        <v>305</v>
+      </c>
+      <c r="E57" s="29" t="s">
+        <v>306</v>
+      </c>
+      <c r="F57" s="29" t="s">
+        <v>307</v>
+      </c>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="B58" s="33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C58" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D58" s="33" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E58" s="33" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F58" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="G58" s="2"/>
+      <c r="H58" s="7" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="18" t="s">
+        <v>399</v>
+      </c>
+      <c r="B59" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C59" s="13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D59" s="13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E59" s="13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F59" s="13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G59" s="2"/>
+      <c r="H59" s="7" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="18" t="s">
+        <v>401</v>
+      </c>
+      <c r="B60" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="C60" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="D60" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="E60" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="F60" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="G60" s="2"/>
+      <c r="H60" s="7" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="B61" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="C61" s="15" t="n">
+        <f aca="false">B61*(1+$B$62)</f>
+        <v>51.5</v>
+      </c>
+      <c r="D61" s="15" t="n">
+        <f aca="false">C61*(1+$B$62)</f>
+        <v>53.045</v>
+      </c>
+      <c r="E61" s="15" t="n">
+        <f aca="false">D61*(1+$B$62)</f>
+        <v>54.63635</v>
+      </c>
+      <c r="F61" s="15" t="n">
+        <f aca="false">E61*(1+$B$62)</f>
+        <v>56.2754405</v>
+      </c>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="18" t="s">
+        <v>403</v>
+      </c>
+      <c r="B62" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C62" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D62" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E62" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F62" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G62" s="2"/>
+      <c r="H62" s="2"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="18" t="s">
+        <v>404</v>
+      </c>
+      <c r="B63" s="12" t="n">
+        <v>69</v>
+      </c>
+      <c r="C63" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="D63" s="12" t="n">
+        <v>260</v>
+      </c>
+      <c r="E63" s="12" t="n">
+        <v>380</v>
+      </c>
+      <c r="F63" s="12" t="n">
+        <v>480</v>
+      </c>
+      <c r="G63" s="2"/>
+      <c r="H63" s="2"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="18" t="s">
+        <v>405</v>
+      </c>
+      <c r="B64" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C64" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D64" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E64" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F64" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G64" s="2"/>
+      <c r="H64" s="2"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="18" t="s">
+        <v>406</v>
+      </c>
+      <c r="B65" s="9" t="n">
+        <v>22000</v>
+      </c>
+      <c r="C65" s="9" t="n">
+        <v>22000</v>
+      </c>
+      <c r="D65" s="9" t="n">
+        <v>22000</v>
+      </c>
+      <c r="E65" s="9" t="n">
+        <v>22000</v>
+      </c>
+      <c r="F65" s="9" t="n">
+        <v>22000</v>
+      </c>
+      <c r="G65" s="2"/>
+      <c r="H65" s="2"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="B66" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C66" s="9" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D66" s="9" t="n">
+        <v>102750</v>
+      </c>
+      <c r="E66" s="9" t="n">
+        <v>191000</v>
+      </c>
+      <c r="F66" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G66" s="2"/>
+      <c r="H66" s="7" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="41" t="s">
+        <v>409</v>
+      </c>
+      <c r="B67" s="42"/>
+      <c r="C67" s="42"/>
+      <c r="D67" s="42"/>
+      <c r="E67" s="42"/>
+      <c r="F67" s="42"/>
+      <c r="G67" s="2"/>
+      <c r="H67" s="42"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="18" t="s">
+        <v>410</v>
+      </c>
+      <c r="B68" s="19" t="n">
+        <f aca="false">B58*Assumptions!$B$8*12</f>
+        <v>378</v>
+      </c>
+      <c r="C68" s="19" t="n">
+        <f aca="false">C58*Assumptions!$B$8*12</f>
+        <v>504</v>
+      </c>
+      <c r="D68" s="19" t="n">
+        <f aca="false">D58*Assumptions!$B$8*12</f>
+        <v>630</v>
+      </c>
+      <c r="E68" s="19" t="n">
+        <f aca="false">E58*Assumptions!$B$8*12</f>
+        <v>882</v>
+      </c>
+      <c r="F68" s="19" t="n">
+        <f aca="false">F58*Assumptions!$B$8*12</f>
+        <v>1008</v>
+      </c>
+      <c r="G68" s="2"/>
+      <c r="H68" s="2"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="16" t="s">
+        <v>411</v>
+      </c>
+      <c r="B69" s="20" t="n">
+        <f aca="false">B68*B59*B60</f>
+        <v>12190.5</v>
+      </c>
+      <c r="C69" s="20" t="n">
+        <f aca="false">C68*C59*C60</f>
+        <v>19504.8</v>
+      </c>
+      <c r="D69" s="20" t="n">
+        <f aca="false">D68*D59*D60</f>
+        <v>25735.5</v>
+      </c>
+      <c r="E69" s="20" t="n">
+        <f aca="false">E68*E59*E60</f>
+        <v>36029.7</v>
+      </c>
+      <c r="F69" s="20" t="n">
+        <f aca="false">F68*F59*F60</f>
+        <v>41176.8</v>
+      </c>
+      <c r="G69" s="2"/>
+      <c r="H69" s="2"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="B70" s="15" t="n">
+        <f aca="false">B69*B61</f>
+        <v>609525</v>
+      </c>
+      <c r="C70" s="15" t="n">
+        <f aca="false">C69*C61</f>
+        <v>1004497.2</v>
+      </c>
+      <c r="D70" s="15" t="n">
+        <f aca="false">D69*D61</f>
+        <v>1365139.5975</v>
+      </c>
+      <c r="E70" s="15" t="n">
+        <f aca="false">E69*E61</f>
+        <v>1968531.299595</v>
+      </c>
+      <c r="F70" s="15" t="n">
+        <f aca="false">F69*F61</f>
+        <v>2317242.5583804</v>
+      </c>
+      <c r="G70" s="2"/>
+      <c r="H70" s="2"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="B71" s="15" t="n">
+        <f aca="false">B68*(1-B59)*Assumptions!$B$10</f>
+        <v>94500</v>
+      </c>
+      <c r="C71" s="15" t="n">
+        <f aca="false">C68*(1-C59)*Assumptions!$B$10</f>
+        <v>50400</v>
+      </c>
+      <c r="D71" s="15" t="n">
+        <f aca="false">D68*(1-D59)*Assumptions!$B$10</f>
+        <v>31500</v>
+      </c>
+      <c r="E71" s="15" t="n">
+        <f aca="false">E68*(1-E59)*Assumptions!$B$10</f>
+        <v>44100</v>
+      </c>
+      <c r="F71" s="15" t="n">
+        <f aca="false">F68*(1-F59)*Assumptions!$B$10</f>
+        <v>50400.0000000001</v>
+      </c>
+      <c r="G71" s="2"/>
+      <c r="H71" s="2"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="B72" s="15" t="n">
+        <f aca="false">B63*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>17181</v>
+      </c>
+      <c r="C72" s="15" t="n">
+        <f aca="false">C63*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>37350</v>
+      </c>
+      <c r="D72" s="15" t="n">
+        <f aca="false">D63*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>64740</v>
+      </c>
+      <c r="E72" s="15" t="n">
+        <f aca="false">E63*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>94620</v>
+      </c>
+      <c r="F72" s="15" t="n">
+        <f aca="false">F63*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>119520</v>
+      </c>
+      <c r="G72" s="2"/>
+      <c r="H72" s="2"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="B73" s="23" t="n">
+        <f aca="false">B70+B71+B72</f>
+        <v>721206</v>
+      </c>
+      <c r="C73" s="23" t="n">
+        <f aca="false">C70+C71+C72</f>
+        <v>1092247.2</v>
+      </c>
+      <c r="D73" s="23" t="n">
+        <f aca="false">D70+D71+D72</f>
+        <v>1461379.5975</v>
+      </c>
+      <c r="E73" s="23" t="n">
+        <f aca="false">E70+E71+E72</f>
+        <v>2107251.299595</v>
+      </c>
+      <c r="F73" s="23" t="n">
+        <f aca="false">F70+F71+F72</f>
+        <v>2487162.5583804</v>
+      </c>
+      <c r="G73" s="2"/>
+      <c r="H73" s="2"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="18" t="s">
+        <v>414</v>
+      </c>
+      <c r="B74" s="15" t="n">
+        <f aca="false">B58*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(B1)-2)</f>
+        <v>250272.18</v>
+      </c>
+      <c r="C74" s="15" t="n">
+        <f aca="false">C58*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(C1)-2)</f>
+        <v>343707.1272</v>
+      </c>
+      <c r="D74" s="15" t="n">
+        <f aca="false">D58*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(D1)-2)</f>
+        <v>442522.92627</v>
+      </c>
+      <c r="E74" s="15" t="n">
+        <f aca="false">E58*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(E1)-2)</f>
+        <v>638118.05968134</v>
+      </c>
+      <c r="F74" s="15" t="n">
+        <f aca="false">F58*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(F1)-2)</f>
+        <v>751156.115967749</v>
+      </c>
+      <c r="G74" s="2"/>
+      <c r="H74" s="2"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="18" t="s">
+        <v>415</v>
+      </c>
+      <c r="B75" s="15" t="n">
+        <f aca="false">(B70+B71)*Assumptions!$B$20+B63/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>145635</v>
+      </c>
+      <c r="C75" s="15" t="n">
+        <f aca="false">(C70+C71)*Assumptions!$B$20+C63/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>221479.44</v>
+      </c>
+      <c r="D75" s="15" t="n">
+        <f aca="false">(D70+D71)*Assumptions!$B$20+D63/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>297527.9195</v>
+      </c>
+      <c r="E75" s="15" t="n">
+        <f aca="false">(E70+E71)*Assumptions!$B$20+E63/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>429126.259919</v>
+      </c>
+      <c r="F75" s="15" t="n">
+        <f aca="false">(F70+F71)*Assumptions!$B$20+F63/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>507128.51167608</v>
+      </c>
+      <c r="G75" s="2"/>
+      <c r="H75" s="2"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="B76" s="23" t="n">
+        <f aca="false">B73-B74-B75</f>
+        <v>325298.82</v>
+      </c>
+      <c r="C76" s="23" t="n">
+        <f aca="false">C73-C74-C75</f>
+        <v>527060.6328</v>
+      </c>
+      <c r="D76" s="23" t="n">
+        <f aca="false">D73-D74-D75</f>
+        <v>721328.75173</v>
+      </c>
+      <c r="E76" s="23" t="n">
+        <f aca="false">E73-E74-E75</f>
+        <v>1040006.97999466</v>
+      </c>
+      <c r="F76" s="23" t="n">
+        <f aca="false">F73-F74-F75</f>
+        <v>1228877.93073657</v>
+      </c>
+      <c r="G76" s="2"/>
+      <c r="H76" s="2"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="B77" s="21" t="n">
+        <f aca="false">IF(B73=0,0,B76/B73)</f>
+        <v>0.451048410578947</v>
+      </c>
+      <c r="C77" s="21" t="n">
+        <f aca="false">IF(C73=0,0,C76/C73)</f>
+        <v>0.482547021223767</v>
+      </c>
+      <c r="D77" s="21" t="n">
+        <f aca="false">IF(D73=0,0,D76/D73)</f>
+        <v>0.493594376823097</v>
+      </c>
+      <c r="E77" s="21" t="n">
+        <f aca="false">IF(E73=0,0,E76/E73)</f>
+        <v>0.49353723506757</v>
+      </c>
+      <c r="F77" s="21" t="n">
+        <f aca="false">IF(F73=0,0,F76/F73)</f>
+        <v>0.494088304198659</v>
+      </c>
+      <c r="G77" s="2"/>
+      <c r="H77" s="2"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="18" t="s">
+        <v>416</v>
+      </c>
+      <c r="B78" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+B58*B65+B66+B73*B64+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,B58-1)</f>
+        <v>216360.45455448</v>
+      </c>
+      <c r="C78" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+C58*C65+C66+C73*C64+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,C58-1)</f>
+        <v>289712.66910896</v>
+      </c>
+      <c r="D78" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+D58*D65+D66+D73*D64+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,D58-1)</f>
+        <v>405719.44353844</v>
+      </c>
+      <c r="E78" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+E58*E65+E66+E73*E64+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,E58-1)</f>
+        <v>575863.337752151</v>
+      </c>
+      <c r="F78" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+F58*F65+F66+F73*F64+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,F58-1)</f>
+        <v>628659.055245901</v>
+      </c>
+      <c r="G78" s="2"/>
+      <c r="H78" s="7" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="16" t="s">
+        <v>418</v>
+      </c>
+      <c r="B79" s="23" t="n">
+        <f aca="false">B76-B78</f>
+        <v>108938.36544552</v>
+      </c>
+      <c r="C79" s="23" t="n">
+        <f aca="false">C76-C78</f>
+        <v>237347.96369104</v>
+      </c>
+      <c r="D79" s="23" t="n">
+        <f aca="false">D76-D78</f>
+        <v>315609.30819156</v>
+      </c>
+      <c r="E79" s="23" t="n">
+        <f aca="false">E76-E78</f>
+        <v>464143.642242509</v>
+      </c>
+      <c r="F79" s="23" t="n">
+        <f aca="false">F76-F78</f>
+        <v>600218.87549067</v>
+      </c>
+      <c r="G79" s="2"/>
+      <c r="H79" s="2"/>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="B80" s="9" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C80" s="9" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D80" s="9" t="n">
+        <v>66000</v>
+      </c>
+      <c r="E80" s="9" t="n">
+        <v>72000</v>
+      </c>
+      <c r="F80" s="9" t="n">
+        <v>72000</v>
+      </c>
+      <c r="G80" s="2"/>
+      <c r="H80" s="7" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="18" t="s">
+        <v>421</v>
+      </c>
+      <c r="B81" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C81" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D81" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E81" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F81" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G81" s="2"/>
+      <c r="H81" s="7" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="18" t="s">
+        <v>423</v>
+      </c>
+      <c r="B82" s="15" t="n">
+        <f aca="false">B80+IF(B80=0,0,B81*MAX(0,B79-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>70893.836544552</v>
+      </c>
+      <c r="C82" s="15" t="n">
+        <f aca="false">C80+IF(C80=0,0,C81*MAX(0,C79-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>83734.796369104</v>
+      </c>
+      <c r="D82" s="15" t="n">
+        <f aca="false">D80+IF(D80=0,0,D81*MAX(0,D79-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>97560.930819156</v>
+      </c>
+      <c r="E82" s="15" t="n">
+        <f aca="false">E80+IF(E80=0,0,E81*MAX(0,E79-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>118414.364224251</v>
+      </c>
+      <c r="F82" s="15" t="n">
+        <f aca="false">F80+IF(F80=0,0,F81*MAX(0,F79-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>132021.887549067</v>
+      </c>
+      <c r="G82" s="2"/>
+      <c r="H82" s="2"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="16" t="s">
+        <v>424</v>
+      </c>
+      <c r="B83" s="23" t="n">
+        <f aca="false">B79-B82</f>
+        <v>38044.5289009678</v>
+      </c>
+      <c r="C83" s="23" t="n">
+        <f aca="false">C79-C82</f>
+        <v>153613.167321936</v>
+      </c>
+      <c r="D83" s="23" t="n">
+        <f aca="false">D79-D82</f>
+        <v>218048.377372404</v>
+      </c>
+      <c r="E83" s="23" t="n">
+        <f aca="false">E79-E82</f>
+        <v>345729.278018258</v>
+      </c>
+      <c r="F83" s="23" t="n">
+        <f aca="false">F79-F82</f>
+        <v>468196.987941603</v>
+      </c>
+      <c r="G83" s="2"/>
+      <c r="H83" s="2"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="18" t="s">
+        <v>425</v>
+      </c>
+      <c r="B84" s="21" t="n">
+        <f aca="false">IF(B73=0,0,B83/B73)</f>
+        <v>0.0527512651045164</v>
+      </c>
+      <c r="C84" s="21" t="n">
+        <f aca="false">IF(C73=0,0,C83/C73)</f>
+        <v>0.1406395615589</v>
+      </c>
+      <c r="D84" s="21" t="n">
+        <f aca="false">IF(D73=0,0,D83/D73)</f>
+        <v>0.149207213338288</v>
+      </c>
+      <c r="E84" s="21" t="n">
+        <f aca="false">IF(E73=0,0,E83/E73)</f>
+        <v>0.164066468049969</v>
+      </c>
+      <c r="F84" s="21" t="n">
+        <f aca="false">IF(F73=0,0,F83/F73)</f>
+        <v>0.188245431069244</v>
+      </c>
+      <c r="G84" s="2"/>
+      <c r="H84" s="2"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="18" t="s">
+        <v>426</v>
+      </c>
+      <c r="B85" s="15" t="n">
+        <f aca="false">MAX(0,B58-1)*'Equipment plan'!$G$10</f>
+        <v>13850</v>
+      </c>
+      <c r="C85" s="15" t="n">
+        <f aca="false">MAX(0,C58-B58)*'Equipment plan'!$G$10</f>
+        <v>13850</v>
+      </c>
+      <c r="D85" s="15" t="n">
+        <f aca="false">MAX(0,D58-C58)*'Equipment plan'!$G$10</f>
+        <v>13850</v>
+      </c>
+      <c r="E85" s="15" t="n">
+        <f aca="false">MAX(0,E58-D58)*'Equipment plan'!$G$10</f>
+        <v>27700</v>
+      </c>
+      <c r="F85" s="15" t="n">
+        <f aca="false">MAX(0,F58-E58)*'Equipment plan'!$G$10</f>
+        <v>13850</v>
+      </c>
+      <c r="G85" s="2"/>
+      <c r="H85" s="2"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="16" t="s">
+        <v>427</v>
+      </c>
+      <c r="B86" s="23" t="n">
+        <f aca="false">Assumptions!$B$39+B83-B85</f>
+        <v>49194.5289009678</v>
+      </c>
+      <c r="C86" s="23" t="n">
+        <f aca="false">B86+C83-C85</f>
+        <v>188957.696222904</v>
+      </c>
+      <c r="D86" s="23" t="n">
+        <f aca="false">C86+D83-D85</f>
+        <v>393156.073595307</v>
+      </c>
+      <c r="E86" s="23" t="n">
+        <f aca="false">D86+E83-E85</f>
+        <v>711185.351613565</v>
+      </c>
+      <c r="F86" s="23" t="n">
+        <f aca="false">E86+F83-F85</f>
+        <v>1165532.33955517</v>
+      </c>
+      <c r="G86" s="2"/>
+      <c r="H86" s="7" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="B87" s="15" t="n">
+        <f aca="false">B83+Assumptions!$B$55*12</f>
+        <v>110044.528900968</v>
+      </c>
+      <c r="C87" s="15" t="n">
+        <f aca="false">C83+Assumptions!$B$55*12</f>
+        <v>225613.167321936</v>
+      </c>
+      <c r="D87" s="15" t="n">
+        <f aca="false">D83+Assumptions!$B$55*12</f>
+        <v>290048.377372404</v>
+      </c>
+      <c r="E87" s="15" t="n">
+        <f aca="false">E83+Assumptions!$B$55*12</f>
+        <v>417729.278018258</v>
+      </c>
+      <c r="F87" s="15" t="n">
+        <f aca="false">F83+Assumptions!$B$55*12</f>
+        <v>540196.987941603</v>
+      </c>
+      <c r="G87" s="2"/>
+      <c r="H87" s="2"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="18" t="s">
+        <v>430</v>
+      </c>
+      <c r="B88" s="15" t="n">
+        <f aca="false">MAX(0,B87)*2.46</f>
+        <v>270709.541096381</v>
+      </c>
+      <c r="C88" s="15" t="n">
+        <f aca="false">MAX(0,C87)*2.46</f>
+        <v>555008.391611962</v>
+      </c>
+      <c r="D88" s="15" t="n">
+        <f aca="false">MAX(0,D87)*2.46</f>
+        <v>713519.008336113</v>
+      </c>
+      <c r="E88" s="15" t="n">
+        <f aca="false">MAX(0,E87)*2.46</f>
+        <v>1027614.02392491</v>
+      </c>
+      <c r="F88" s="15" t="n">
+        <f aca="false">MAX(0,F87)*2.46</f>
+        <v>1328884.59033634</v>
+      </c>
+      <c r="G88" s="2"/>
+      <c r="H88" s="7" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="2"/>
+      <c r="B89" s="2"/>
+      <c r="C89" s="2"/>
+      <c r="D89" s="2"/>
+      <c r="E89" s="2"/>
+      <c r="F89" s="2"/>
+      <c r="G89" s="2"/>
+      <c r="H89" s="2"/>
+    </row>
+    <row r="90" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="B90" s="5"/>
+      <c r="C90" s="5"/>
+      <c r="D90" s="5"/>
+      <c r="E90" s="5"/>
+      <c r="F90" s="5"/>
+      <c r="G90" s="2"/>
+      <c r="H90" s="40" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="B91" s="29" t="s">
+        <v>151</v>
+      </c>
+      <c r="C91" s="29" t="s">
+        <v>152</v>
+      </c>
+      <c r="D91" s="29" t="s">
+        <v>305</v>
+      </c>
+      <c r="E91" s="29" t="s">
+        <v>306</v>
+      </c>
+      <c r="F91" s="29" t="s">
+        <v>307</v>
+      </c>
+      <c r="G91" s="2"/>
+      <c r="H91" s="2"/>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="B92" s="33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C92" s="33" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D92" s="33" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E92" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="F92" s="33" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G92" s="2"/>
+      <c r="H92" s="7" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="18" t="s">
+        <v>399</v>
+      </c>
+      <c r="B93" s="13" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C93" s="13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D93" s="13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E93" s="13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F93" s="13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G93" s="2"/>
+      <c r="H93" s="7" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="18" t="s">
+        <v>401</v>
+      </c>
+      <c r="B94" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="C94" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="D94" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="E94" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="F94" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="G94" s="2"/>
+      <c r="H94" s="7" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="B95" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="C95" s="15" t="n">
+        <f aca="false">B95*(1+$B$96)</f>
+        <v>53.56</v>
+      </c>
+      <c r="D95" s="15" t="n">
+        <f aca="false">C95*(1+$B$96)</f>
+        <v>55.1668</v>
+      </c>
+      <c r="E95" s="15" t="n">
+        <f aca="false">D95*(1+$B$96)</f>
+        <v>56.821804</v>
+      </c>
+      <c r="F95" s="15" t="n">
+        <f aca="false">E95*(1+$B$96)</f>
+        <v>58.52645812</v>
+      </c>
+      <c r="G95" s="2"/>
+      <c r="H95" s="2"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="18" t="s">
+        <v>403</v>
+      </c>
+      <c r="B96" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C96" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D96" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E96" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F96" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="G96" s="2"/>
+      <c r="H96" s="2"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="18" t="s">
+        <v>404</v>
+      </c>
+      <c r="B97" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="C97" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="D97" s="12" t="n">
+        <v>340</v>
+      </c>
+      <c r="E97" s="12" t="n">
+        <v>480</v>
+      </c>
+      <c r="F97" s="12" t="n">
+        <v>620</v>
+      </c>
+      <c r="G97" s="2"/>
+      <c r="H97" s="2"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="18" t="s">
+        <v>405</v>
+      </c>
+      <c r="B98" s="13" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="C98" s="13" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="D98" s="13" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="E98" s="13" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="F98" s="13" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="G98" s="2"/>
+      <c r="H98" s="2"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="18" t="s">
+        <v>406</v>
+      </c>
+      <c r="B99" s="9" t="n">
+        <v>22000</v>
+      </c>
+      <c r="C99" s="9" t="n">
+        <v>22000</v>
+      </c>
+      <c r="D99" s="9" t="n">
+        <v>22000</v>
+      </c>
+      <c r="E99" s="9" t="n">
+        <v>22000</v>
+      </c>
+      <c r="F99" s="9" t="n">
+        <v>22000</v>
+      </c>
+      <c r="G99" s="2"/>
+      <c r="H99" s="2"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="B100" s="9" t="n">
+        <v>12000</v>
+      </c>
+      <c r="C100" s="9" t="n">
+        <v>54000</v>
+      </c>
+      <c r="D100" s="9" t="n">
+        <v>191000</v>
+      </c>
+      <c r="E100" s="9" t="n">
+        <v>265000</v>
+      </c>
+      <c r="F100" s="9" t="n">
+        <v>290000</v>
+      </c>
+      <c r="G100" s="2"/>
+      <c r="H100" s="7" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="41" t="s">
+        <v>409</v>
+      </c>
+      <c r="B101" s="42"/>
+      <c r="C101" s="42"/>
+      <c r="D101" s="42"/>
+      <c r="E101" s="42"/>
+      <c r="F101" s="42"/>
+      <c r="G101" s="2"/>
+      <c r="H101" s="42"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="18" t="s">
+        <v>410</v>
+      </c>
+      <c r="B102" s="19" t="n">
+        <f aca="false">B92*Assumptions!$B$8*12</f>
+        <v>378</v>
+      </c>
+      <c r="C102" s="19" t="n">
+        <f aca="false">C92*Assumptions!$B$8*12</f>
+        <v>630</v>
+      </c>
+      <c r="D102" s="19" t="n">
+        <f aca="false">D92*Assumptions!$B$8*12</f>
+        <v>882</v>
+      </c>
+      <c r="E102" s="19" t="n">
+        <f aca="false">E92*Assumptions!$B$8*12</f>
+        <v>1008</v>
+      </c>
+      <c r="F102" s="19" t="n">
+        <f aca="false">F92*Assumptions!$B$8*12</f>
+        <v>1134</v>
+      </c>
+      <c r="G102" s="2"/>
+      <c r="H102" s="2"/>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="16" t="s">
+        <v>411</v>
+      </c>
+      <c r="B103" s="20" t="n">
+        <f aca="false">B102*B93*B94</f>
+        <v>15422.4</v>
+      </c>
+      <c r="C103" s="20" t="n">
+        <f aca="false">C102*C93*C94</f>
+        <v>28728</v>
+      </c>
+      <c r="D103" s="20" t="n">
+        <f aca="false">D102*D93*D94</f>
+        <v>40219.2</v>
+      </c>
+      <c r="E103" s="20" t="n">
+        <f aca="false">E102*E93*E94</f>
+        <v>45964.8</v>
+      </c>
+      <c r="F103" s="20" t="n">
+        <f aca="false">F102*F93*F94</f>
+        <v>51710.4</v>
+      </c>
+      <c r="G103" s="2"/>
+      <c r="H103" s="2"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="B104" s="15" t="n">
+        <f aca="false">B103*B95</f>
+        <v>801964.8</v>
+      </c>
+      <c r="C104" s="15" t="n">
+        <f aca="false">C103*C95</f>
+        <v>1538671.68</v>
+      </c>
+      <c r="D104" s="15" t="n">
+        <f aca="false">D103*D95</f>
+        <v>2218764.56256</v>
+      </c>
+      <c r="E104" s="15" t="n">
+        <f aca="false">E103*E95</f>
+        <v>2611802.8564992</v>
+      </c>
+      <c r="F104" s="15" t="n">
+        <f aca="false">F103*F95</f>
+        <v>3026426.55996845</v>
+      </c>
+      <c r="G104" s="2"/>
+      <c r="H104" s="2"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="18" t="s">
+        <v>413</v>
+      </c>
+      <c r="B105" s="15" t="n">
+        <f aca="false">B102*(1-B93)*Assumptions!$B$10</f>
+        <v>56700</v>
+      </c>
+      <c r="C105" s="15" t="n">
+        <f aca="false">C102*(1-C93)*Assumptions!$B$10</f>
+        <v>31500</v>
+      </c>
+      <c r="D105" s="15" t="n">
+        <f aca="false">D102*(1-D93)*Assumptions!$B$10</f>
+        <v>44100</v>
+      </c>
+      <c r="E105" s="15" t="n">
+        <f aca="false">E102*(1-E93)*Assumptions!$B$10</f>
+        <v>50400.0000000001</v>
+      </c>
+      <c r="F105" s="15" t="n">
+        <f aca="false">F102*(1-F93)*Assumptions!$B$10</f>
+        <v>56700.0000000001</v>
+      </c>
+      <c r="G105" s="2"/>
+      <c r="H105" s="2"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="B106" s="15" t="n">
+        <f aca="false">B97*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>22410</v>
+      </c>
+      <c r="C106" s="15" t="n">
+        <f aca="false">C97*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>49800</v>
+      </c>
+      <c r="D106" s="15" t="n">
+        <f aca="false">D97*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>84660</v>
+      </c>
+      <c r="E106" s="15" t="n">
+        <f aca="false">E97*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>119520</v>
+      </c>
+      <c r="F106" s="15" t="n">
+        <f aca="false">F97*Assumptions!$B$28/Assumptions!$B$29</f>
+        <v>154380</v>
+      </c>
+      <c r="G106" s="2"/>
+      <c r="H106" s="2"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="B107" s="23" t="n">
+        <f aca="false">B104+B105+B106</f>
+        <v>881074.8</v>
+      </c>
+      <c r="C107" s="23" t="n">
+        <f aca="false">C104+C105+C106</f>
+        <v>1619971.68</v>
+      </c>
+      <c r="D107" s="23" t="n">
+        <f aca="false">D104+D105+D106</f>
+        <v>2347524.56256</v>
+      </c>
+      <c r="E107" s="23" t="n">
+        <f aca="false">E104+E105+E106</f>
+        <v>2781722.8564992</v>
+      </c>
+      <c r="F107" s="23" t="n">
+        <f aca="false">F104+F105+F106</f>
+        <v>3237506.55996845</v>
+      </c>
+      <c r="G107" s="2"/>
+      <c r="H107" s="2"/>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="18" t="s">
+        <v>414</v>
+      </c>
+      <c r="B108" s="15" t="n">
+        <f aca="false">B92*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(B1)-2)</f>
+        <v>250272.18</v>
+      </c>
+      <c r="C108" s="15" t="n">
+        <f aca="false">C92*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(C1)-2)</f>
+        <v>429633.909</v>
+      </c>
+      <c r="D108" s="15" t="n">
+        <f aca="false">D92*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(D1)-2)</f>
+        <v>619532.096778</v>
+      </c>
+      <c r="E108" s="15" t="n">
+        <f aca="false">E92*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(E1)-2)</f>
+        <v>729277.78249296</v>
+      </c>
+      <c r="F108" s="15" t="n">
+        <f aca="false">F92*(Assumptions!$B$24*Assumptions!$B$25*Assumptions!$B$21+Assumptions!$B$25*Assumptions!$B$22)*(1+Assumptions!$B$23)*12*1.03^MAX(0,COLUMN(F1)-2)</f>
+        <v>845050.630463718</v>
+      </c>
+      <c r="G108" s="2"/>
+      <c r="H108" s="2"/>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="18" t="s">
+        <v>415</v>
+      </c>
+      <c r="B109" s="15" t="n">
+        <f aca="false">(B104+B105)*Assumptions!$B$20+B97/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>178032.96</v>
+      </c>
+      <c r="C109" s="15" t="n">
+        <f aca="false">(C104+C105)*Assumptions!$B$20+C97/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>328034.336</v>
+      </c>
+      <c r="D109" s="15" t="n">
+        <f aca="false">(D104+D105)*Assumptions!$B$20+D97/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>476372.912512</v>
+      </c>
+      <c r="E109" s="15" t="n">
+        <f aca="false">(E104+E105)*Assumptions!$B$20+E97/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>566040.57129984</v>
+      </c>
+      <c r="F109" s="15" t="n">
+        <f aca="false">(F104+F105)*Assumptions!$B$20+F97/Assumptions!$B$29*Assumptions!$B$34</f>
+        <v>660025.31199369</v>
+      </c>
+      <c r="G109" s="2"/>
+      <c r="H109" s="2"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="B110" s="23" t="n">
+        <f aca="false">B107-B108-B109</f>
+        <v>452769.66</v>
+      </c>
+      <c r="C110" s="23" t="n">
+        <f aca="false">C107-C108-C109</f>
+        <v>862303.435</v>
+      </c>
+      <c r="D110" s="23" t="n">
+        <f aca="false">D107-D108-D109</f>
+        <v>1251619.55327</v>
+      </c>
+      <c r="E110" s="23" t="n">
+        <f aca="false">E107-E108-E109</f>
+        <v>1486404.5027064</v>
+      </c>
+      <c r="F110" s="23" t="n">
+        <f aca="false">F107-F108-F109</f>
+        <v>1732430.61751104</v>
+      </c>
+      <c r="G110" s="2"/>
+      <c r="H110" s="2"/>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="B111" s="21" t="n">
+        <f aca="false">IF(B107=0,0,B110/B107)</f>
+        <v>0.513883338849324</v>
+      </c>
+      <c r="C111" s="21" t="n">
+        <f aca="false">IF(C107=0,0,C110/C107)</f>
+        <v>0.532295376299418</v>
+      </c>
+      <c r="D111" s="21" t="n">
+        <f aca="false">IF(D107=0,0,D110/D107)</f>
+        <v>0.533165690034398</v>
+      </c>
+      <c r="E111" s="21" t="n">
+        <f aca="false">IF(E107=0,0,E110/E107)</f>
+        <v>0.53434672660994</v>
+      </c>
+      <c r="F111" s="21" t="n">
+        <f aca="false">IF(F107=0,0,F110/F107)</f>
+        <v>0.535112619981201</v>
+      </c>
+      <c r="G111" s="2"/>
+      <c r="H111" s="2"/>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="18" t="s">
+        <v>416</v>
+      </c>
+      <c r="B112" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+B92*B99+B100+B107*B98+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,B92-1)</f>
+        <v>231948.52055448</v>
+      </c>
+      <c r="C112" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+C92*C99+C100+C107*C98+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,C92-1)</f>
+        <v>356799.18926344</v>
+      </c>
+      <c r="D112" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+D92*D99+D100+D107*D98+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,D92-1)</f>
+        <v>576139.378087601</v>
+      </c>
+      <c r="E112" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+E92*E99+E100+E107*E98+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,E92-1)</f>
+        <v>694478.455869345</v>
+      </c>
+      <c r="F112" s="15" t="n">
+        <f aca="false">(Assumptions!$B$55+Assumptions!$B$57+Assumptions!$B$58+Assumptions!$B$59+Assumptions!$B$60)*12+F92*F99+F100+F107*F98+Assumptions!$B$61*Assumptions!$B$62*12+'Equipment plan'!$H$10*12*MAX(0,F92-1)</f>
+        <v>764788.877079941</v>
+      </c>
+      <c r="G112" s="2"/>
+      <c r="H112" s="7" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="16" t="s">
+        <v>418</v>
+      </c>
+      <c r="B113" s="23" t="n">
+        <f aca="false">B110-B112</f>
+        <v>220821.13944552</v>
+      </c>
+      <c r="C113" s="23" t="n">
+        <f aca="false">C110-C112</f>
+        <v>505504.24573656</v>
+      </c>
+      <c r="D113" s="23" t="n">
+        <f aca="false">D110-D112</f>
+        <v>675480.175182399</v>
+      </c>
+      <c r="E113" s="23" t="n">
+        <f aca="false">E110-E112</f>
+        <v>791926.046837055</v>
+      </c>
+      <c r="F113" s="23" t="n">
+        <f aca="false">F110-F112</f>
+        <v>967641.740431099</v>
+      </c>
+      <c r="G113" s="2"/>
+      <c r="H113" s="2"/>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="B114" s="9" t="n">
+        <v>60000</v>
+      </c>
+      <c r="C114" s="9" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D114" s="9" t="n">
+        <v>66000</v>
+      </c>
+      <c r="E114" s="9" t="n">
+        <v>72000</v>
+      </c>
+      <c r="F114" s="9" t="n">
+        <v>72000</v>
+      </c>
+      <c r="G114" s="2"/>
+      <c r="H114" s="7" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="18" t="s">
+        <v>421</v>
+      </c>
+      <c r="B115" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C115" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D115" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E115" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F115" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G115" s="2"/>
+      <c r="H115" s="7" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="18" t="s">
+        <v>423</v>
+      </c>
+      <c r="B116" s="15" t="n">
+        <f aca="false">B114+IF(B114=0,0,B115*MAX(0,B113-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>82082.113944552</v>
+      </c>
+      <c r="C116" s="15" t="n">
+        <f aca="false">C114+IF(C114=0,0,C115*MAX(0,C113-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>110550.424573656</v>
+      </c>
+      <c r="D116" s="15" t="n">
+        <f aca="false">D114+IF(D114=0,0,D115*MAX(0,D113-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>133548.01751824</v>
+      </c>
+      <c r="E116" s="15" t="n">
+        <f aca="false">E114+IF(E114=0,0,E115*MAX(0,E113-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>151192.604683706</v>
+      </c>
+      <c r="F116" s="15" t="n">
+        <f aca="false">F114+IF(F114=0,0,F115*MAX(0,F113-MAX(0,'5-year plan'!$B$44)))</f>
+        <v>168764.17404311</v>
+      </c>
+      <c r="G116" s="2"/>
+      <c r="H116" s="2"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="16" t="s">
+        <v>424</v>
+      </c>
+      <c r="B117" s="23" t="n">
+        <f aca="false">B113-B116</f>
+        <v>138739.025500968</v>
+      </c>
+      <c r="C117" s="23" t="n">
+        <f aca="false">C113-C116</f>
+        <v>394953.821162904</v>
+      </c>
+      <c r="D117" s="23" t="n">
+        <f aca="false">D113-D116</f>
+        <v>541932.157664159</v>
+      </c>
+      <c r="E117" s="23" t="n">
+        <f aca="false">E113-E116</f>
+        <v>640733.442153349</v>
+      </c>
+      <c r="F117" s="23" t="n">
+        <f aca="false">F113-F116</f>
+        <v>798877.56638799</v>
+      </c>
+      <c r="G117" s="2"/>
+      <c r="H117" s="2"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="18" t="s">
+        <v>425</v>
+      </c>
+      <c r="B118" s="21" t="n">
+        <f aca="false">IF(B107=0,0,B117/B107)</f>
+        <v>0.157465660691882</v>
+      </c>
+      <c r="C118" s="21" t="n">
+        <f aca="false">IF(C107=0,0,C117/C107)</f>
+        <v>0.243802917075009</v>
+      </c>
+      <c r="D118" s="21" t="n">
+        <f aca="false">IF(D107=0,0,D117/D107)</f>
+        <v>0.230852603762824</v>
+      </c>
+      <c r="E118" s="21" t="n">
+        <f aca="false">IF(E107=0,0,E117/E107)</f>
+        <v>0.23033690817054</v>
+      </c>
+      <c r="F118" s="21" t="n">
+        <f aca="false">IF(F107=0,0,F117/F107)</f>
+        <v>0.246757049473214</v>
+      </c>
+      <c r="G118" s="2"/>
+      <c r="H118" s="2"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="18" t="s">
+        <v>426</v>
+      </c>
+      <c r="B119" s="15" t="n">
+        <f aca="false">MAX(0,B92-1)*'Equipment plan'!$G$10</f>
+        <v>13850</v>
+      </c>
+      <c r="C119" s="15" t="n">
+        <f aca="false">MAX(0,C92-B92)*'Equipment plan'!$G$10</f>
+        <v>27700</v>
+      </c>
+      <c r="D119" s="15" t="n">
+        <f aca="false">MAX(0,D92-C92)*'Equipment plan'!$G$10</f>
+        <v>27700</v>
+      </c>
+      <c r="E119" s="15" t="n">
+        <f aca="false">MAX(0,E92-D92)*'Equipment plan'!$G$10</f>
+        <v>13850</v>
+      </c>
+      <c r="F119" s="15" t="n">
+        <f aca="false">MAX(0,F92-E92)*'Equipment plan'!$G$10</f>
+        <v>13850</v>
+      </c>
+      <c r="G119" s="2"/>
+      <c r="H119" s="2"/>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="16" t="s">
+        <v>427</v>
+      </c>
+      <c r="B120" s="23" t="n">
+        <f aca="false">Assumptions!$B$39+B117-B119</f>
+        <v>149889.025500968</v>
+      </c>
+      <c r="C120" s="23" t="n">
+        <f aca="false">B120+C117-C119</f>
+        <v>517142.846663872</v>
+      </c>
+      <c r="D120" s="23" t="n">
+        <f aca="false">C120+D117-D119</f>
+        <v>1031375.00432803</v>
+      </c>
+      <c r="E120" s="23" t="n">
+        <f aca="false">D120+E117-E119</f>
+        <v>1658258.44648138</v>
+      </c>
+      <c r="F120" s="23" t="n">
+        <f aca="false">E120+F117-F119</f>
+        <v>2443286.01286937</v>
+      </c>
+      <c r="G120" s="2"/>
+      <c r="H120" s="7" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="B121" s="15" t="n">
+        <f aca="false">B117+Assumptions!$B$55*12</f>
+        <v>210739.025500968</v>
+      </c>
+      <c r="C121" s="15" t="n">
+        <f aca="false">C117+Assumptions!$B$55*12</f>
+        <v>466953.821162904</v>
+      </c>
+      <c r="D121" s="15" t="n">
+        <f aca="false">D117+Assumptions!$B$55*12</f>
+        <v>613932.157664159</v>
+      </c>
+      <c r="E121" s="15" t="n">
+        <f aca="false">E117+Assumptions!$B$55*12</f>
+        <v>712733.442153349</v>
+      </c>
+      <c r="F121" s="15" t="n">
+        <f aca="false">F117+Assumptions!$B$55*12</f>
+        <v>870877.56638799</v>
+      </c>
+      <c r="G121" s="2"/>
+      <c r="H121" s="2"/>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="18" t="s">
+        <v>430</v>
+      </c>
+      <c r="B122" s="15" t="n">
+        <f aca="false">MAX(0,B121)*2.46</f>
+        <v>518418.002732381</v>
+      </c>
+      <c r="C122" s="15" t="n">
+        <f aca="false">MAX(0,C121)*2.46</f>
+        <v>1148706.40006074</v>
+      </c>
+      <c r="D122" s="15" t="n">
+        <f aca="false">MAX(0,D121)*2.46</f>
+        <v>1510273.10785383</v>
+      </c>
+      <c r="E122" s="15" t="n">
+        <f aca="false">MAX(0,E121)*2.46</f>
+        <v>1753324.26769724</v>
+      </c>
+      <c r="F122" s="15" t="n">
+        <f aca="false">MAX(0,F121)*2.46</f>
+        <v>2142358.81331445</v>
+      </c>
+      <c r="G122" s="2"/>
+      <c r="H122" s="7" t="s">
+        <v>431</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection sheet="true" password="ef11" formatCells="false" formatColumns="false" formatRows="false"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -12123,7 +15202,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>377</v>
+        <v>436</v>
       </c>
       <c r="B1" s="2"/>
     </row>
@@ -12132,107 +15211,107 @@
       <c r="B2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="39" t="s">
-        <v>378</v>
-      </c>
-      <c r="B3" s="40" t="s">
-        <v>379</v>
+      <c r="A3" s="43" t="s">
+        <v>437</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>438</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="39" t="s">
-        <v>380</v>
-      </c>
-      <c r="B4" s="40" t="s">
-        <v>381</v>
+      <c r="A4" s="43" t="s">
+        <v>439</v>
+      </c>
+      <c r="B4" s="44" t="s">
+        <v>440</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="39" t="s">
-        <v>382</v>
-      </c>
-      <c r="B5" s="40" t="s">
-        <v>383</v>
+      <c r="A5" s="43" t="s">
+        <v>441</v>
+      </c>
+      <c r="B5" s="44" t="s">
+        <v>442</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="39" t="s">
-        <v>384</v>
-      </c>
-      <c r="B6" s="40" t="s">
-        <v>385</v>
+      <c r="A6" s="43" t="s">
+        <v>443</v>
+      </c>
+      <c r="B6" s="44" t="s">
+        <v>444</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="39" t="s">
-        <v>386</v>
-      </c>
-      <c r="B7" s="40" t="s">
-        <v>387</v>
+      <c r="A7" s="43" t="s">
+        <v>445</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>446</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="39" t="s">
-        <v>388</v>
-      </c>
-      <c r="B8" s="40" t="s">
-        <v>389</v>
+      <c r="A8" s="43" t="s">
+        <v>447</v>
+      </c>
+      <c r="B8" s="44" t="s">
+        <v>448</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="39" t="s">
-        <v>390</v>
-      </c>
-      <c r="B9" s="40" t="s">
-        <v>391</v>
+      <c r="A9" s="43" t="s">
+        <v>449</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>450</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="39" t="s">
-        <v>392</v>
-      </c>
-      <c r="B10" s="40" t="s">
-        <v>393</v>
+      <c r="A10" s="43" t="s">
+        <v>451</v>
+      </c>
+      <c r="B10" s="44" t="s">
+        <v>452</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="39" t="s">
-        <v>394</v>
-      </c>
-      <c r="B11" s="40" t="s">
-        <v>395</v>
+      <c r="A11" s="43" t="s">
+        <v>453</v>
+      </c>
+      <c r="B11" s="44" t="s">
+        <v>454</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="39" t="s">
-        <v>396</v>
-      </c>
-      <c r="B12" s="40" t="s">
-        <v>397</v>
+      <c r="A12" s="43" t="s">
+        <v>455</v>
+      </c>
+      <c r="B12" s="44" t="s">
+        <v>456</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="39" t="s">
-        <v>398</v>
-      </c>
-      <c r="B13" s="40" t="s">
-        <v>399</v>
+      <c r="A13" s="43" t="s">
+        <v>457</v>
+      </c>
+      <c r="B13" s="44" t="s">
+        <v>458</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="39" t="s">
-        <v>400</v>
-      </c>
-      <c r="B14" s="40" t="s">
-        <v>401</v>
+      <c r="A14" s="43" t="s">
+        <v>459</v>
+      </c>
+      <c r="B14" s="44" t="s">
+        <v>460</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="39" t="s">
-        <v>402</v>
-      </c>
-      <c r="B15" s="40" t="s">
-        <v>403</v>
+      <c r="A15" s="43" t="s">
+        <v>461</v>
+      </c>
+      <c r="B15" s="44" t="s">
+        <v>462</v>
       </c>
     </row>
   </sheetData>

</xml_diff>